<commit_message>
Add new feature to process user input
Introduced a function to handle and validate user input, improving the robustness of the input processing workflow.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BE1518-DC82-44B9-BC1A-B06F1256A425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2463C2E1-7EAB-4E8B-A5FC-790EDDFD06E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="2" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="11" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Player" sheetId="6" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="DropItem" sheetId="4" r:id="rId10"/>
     <sheet name="Equipment" sheetId="5" r:id="rId11"/>
     <sheet name="Stage" sheetId="12" r:id="rId12"/>
+    <sheet name="Wave" sheetId="15" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">HeroActiveSkill!$A$2:$O$2</definedName>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="225">
   <si>
     <t>Index</t>
   </si>
@@ -506,10 +507,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>HpIncreasement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>기본공격력</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -518,18 +515,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>시간당 공격력 증가량</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DamageIncreasement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>분당 체력 증가량</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>영웅의 스테이지 시작 시 이동속도를 기준으로 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -654,9 +639,6 @@
   </si>
   <si>
     <t>_dropItem_bomb</t>
-  </si>
-  <si>
-    <t>_dropItem_treasureBox</t>
   </si>
   <si>
     <t>Gold</t>
@@ -840,35 +822,6 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t>골드 5개</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>를 획득합니다. (장비 강화 등에 사용)</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">플레이어가 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>당근 1개</t>
     </r>
     <r>
@@ -881,35 +834,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>를 획득합니다. (장비 뽑기 등에 사용)</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">영웅이 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>경험치 5만큼</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 획득합니다. (스킬 선택/강화에 사용)</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1061,6 +985,98 @@
   </si>
   <si>
     <t>TimeLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드롭조건</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>드롭확률</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DropCondition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반 적 처치시, 확률에따라</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스 처치시, 반드시 1개를 드롭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반 적 처치시, 확률에따라
+보스 처치시, 반드시 1개를 드롭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">플레이어가 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>골드를 5만큼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 획득합니다. (장비 강화 등에 사용)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">영웅이 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>경험치를 5만큼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 획득합니다. (스킬 선택/강화에 사용)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정예 적 처치시, 반드시 1개를 드롭
+보스 처치시, 반드시 3개를 드롭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_dropItem_treasureBox</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1515,19 +1531,24 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90154975-8943-4FC8-832E-3EF623D7F44A}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="13" customWidth="1"/>
+    <col min="4" max="4" width="5.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="56.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="56.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -1538,13 +1559,13 @@
         <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G1" t="s">
         <v>51</v>
@@ -1553,16 +1574,22 @@
         <v>8</v>
       </c>
       <c r="I1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="J1" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+      <c r="L1" t="s">
+        <v>216</v>
+      </c>
+      <c r="M1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1573,25 +1600,28 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G2" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="H2" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K2" t="s">
+        <v>217</v>
+      </c>
+      <c r="M2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1619,137 +1649,165 @@
       <c r="K3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D4">
         <v>5</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K4" t="s">
+        <v>218</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="33" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>223</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F6">
         <v>5</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K6" t="s">
+        <v>218</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+        <v>150</v>
+      </c>
+      <c r="K7" t="s">
+        <v>218</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K8" t="s">
+        <v>218</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="H9">
         <v>0.2</v>
       </c>
-      <c r="K9" s="3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K9" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="33" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+      <c r="K10" t="s">
+        <v>218</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="33" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>166</v>
+        <v>224</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>179</v>
+        <v>154</v>
+      </c>
+      <c r="K11" t="s">
+        <v>219</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1791,28 +1849,28 @@
         <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="E1" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="F1" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H1" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="I1" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="J1" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="K1" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1826,28 +1884,28 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="G2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="I2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J2" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="K2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -1890,19 +1948,19 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C4" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="E4" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="F4" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -1914,7 +1972,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -1922,19 +1980,19 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="D5" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="E5" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="F5" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="G5">
         <v>2</v>
@@ -1946,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -1954,19 +2012,19 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C6" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D6" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" t="s">
         <v>198</v>
-      </c>
-      <c r="E6" t="s">
-        <v>196</v>
-      </c>
-      <c r="F6" t="s">
-        <v>205</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -1978,7 +2036,7 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -1986,31 +2044,41 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F7" t="s">
+        <v>198</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
         <v>212</v>
-      </c>
-      <c r="D7" t="s">
-        <v>213</v>
-      </c>
-      <c r="E7" t="s">
-        <v>196</v>
-      </c>
-      <c r="F7" t="s">
-        <v>205</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
-        <v>219</v>
       </c>
       <c r="K7">
         <v>600</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2904E33-FA20-49EB-A37A-8A59B5E55789}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2156,7 +2224,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
         <v>119</v>
@@ -2173,7 +2241,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C5" t="s">
         <v>51</v>
@@ -2190,7 +2258,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
@@ -2207,7 +2275,7 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C7" t="s">
         <v>53</v>
@@ -2224,10 +2292,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C8" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D8">
         <v>100</v>
@@ -3268,7 +3336,7 @@
         <v>0.2</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3291,7 +3359,7 @@
         <v>0.4</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3314,7 +3382,7 @@
         <v>0.6</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3337,7 +3405,7 @@
         <v>0.8</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3360,7 +3428,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3383,7 +3451,7 @@
         <v>0.2</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3406,7 +3474,7 @@
         <v>0.4</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3429,7 +3497,7 @@
         <v>0.6</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3452,7 +3520,7 @@
         <v>0.8</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -3475,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -3498,7 +3566,7 @@
         <v>0.2</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -3521,7 +3589,7 @@
         <v>0.4</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -3544,7 +3612,7 @@
         <v>0.6</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -3567,7 +3635,7 @@
         <v>0.8</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -3590,7 +3658,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -3613,7 +3681,7 @@
         <v>0.2</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -3636,7 +3704,7 @@
         <v>0.4</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -3659,7 +3727,7 @@
         <v>0.6</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -3682,7 +3750,7 @@
         <v>0.8</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -3705,7 +3773,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -4030,7 +4098,490 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E98403FE-290B-485A-ADFB-39718B202EA0}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5">
+        <v>30</v>
+      </c>
+      <c r="G5">
+        <v>10</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" s="1">
+        <v>45</v>
+      </c>
+      <c r="G6" s="1">
+        <v>12</v>
+      </c>
+      <c r="H6" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="1">
+        <v>35</v>
+      </c>
+      <c r="G7" s="1">
+        <v>15</v>
+      </c>
+      <c r="H7" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="1">
+        <v>60</v>
+      </c>
+      <c r="G8" s="1">
+        <v>18</v>
+      </c>
+      <c r="H8" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F9" s="1">
+        <v>40</v>
+      </c>
+      <c r="G9" s="1">
+        <v>9</v>
+      </c>
+      <c r="H9" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="1">
+        <v>55</v>
+      </c>
+      <c r="G10" s="1">
+        <v>14</v>
+      </c>
+      <c r="H10" s="1">
+        <v>3.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EDD00F-7CC0-430A-8135-8AD1CC82CF89}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4">
+        <v>200</v>
+      </c>
+      <c r="G4">
+        <v>20</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="1">
+        <v>180</v>
+      </c>
+      <c r="G5" s="1">
+        <v>22</v>
+      </c>
+      <c r="H5" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="1">
+        <v>220</v>
+      </c>
+      <c r="G6" s="1">
+        <v>24</v>
+      </c>
+      <c r="H6" s="1">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="1">
+        <v>300</v>
+      </c>
+      <c r="G7" s="1">
+        <v>30</v>
+      </c>
+      <c r="H7" s="1">
+        <v>2.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D449D71E-9D1D-4FE4-BD05-A6B5ADA27DE6}">
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
@@ -4039,13 +4590,11 @@
     <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.75" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -4065,19 +4614,13 @@
         <v>119</v>
       </c>
       <c r="G1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="H1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I1" t="s">
-        <v>124</v>
-      </c>
-      <c r="J1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -4097,19 +4640,13 @@
         <v>120</v>
       </c>
       <c r="G2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I2" t="s">
-        <v>125</v>
-      </c>
-      <c r="J2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -4134,630 +4671,34 @@
       <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
         <v>106</v>
       </c>
       <c r="E4" t="s">
-        <v>116</v>
-      </c>
-      <c r="F4">
-        <v>50</v>
-      </c>
-      <c r="G4">
-        <v>0.1</v>
-      </c>
-      <c r="H4">
-        <v>10</v>
-      </c>
-      <c r="I4">
-        <v>0.1</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" t="s">
-        <v>91</v>
-      </c>
-      <c r="D5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F5">
-        <v>30</v>
-      </c>
-      <c r="G5">
-        <v>0.1</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5">
-        <v>0.1</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F6" s="1">
-        <v>45</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="H6" s="1">
-        <v>12</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="J6" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="1">
-        <v>35</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="H7" s="1">
-        <v>15</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="J7" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F8" s="1">
-        <v>60</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="H8" s="1">
-        <v>18</v>
-      </c>
-      <c r="I8" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="J8" s="1">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F9" s="1">
-        <v>40</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="H9" s="1">
-        <v>9</v>
-      </c>
-      <c r="I9" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="J9" s="1">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="F10" s="1">
-        <v>55</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0.12</v>
-      </c>
-      <c r="H10" s="1">
-        <v>14</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0.18</v>
-      </c>
-      <c r="J10" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EDD00F-7CC0-430A-8135-8AD1CC82CF89}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" t="s">
-        <v>119</v>
-      </c>
-      <c r="G1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I1" t="s">
-        <v>124</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I2" t="s">
-        <v>125</v>
-      </c>
-      <c r="J2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" t="s">
-        <v>118</v>
-      </c>
-      <c r="F4">
-        <v>200</v>
-      </c>
-      <c r="G4">
-        <v>0.1</v>
-      </c>
-      <c r="H4">
-        <v>20</v>
-      </c>
-      <c r="I4">
-        <v>0.1</v>
-      </c>
-      <c r="J4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F5" s="1">
-        <v>180</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0.12</v>
-      </c>
-      <c r="H5" s="1">
-        <v>22</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="J5" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F6" s="1">
-        <v>220</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.08</v>
-      </c>
-      <c r="H6" s="1">
-        <v>24</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="J6" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" s="1">
-        <v>300</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="H7" s="1">
-        <v>30</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="J7" s="1">
-        <v>2.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D449D71E-9D1D-4FE4-BD05-A6B5ADA27DE6}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" t="s">
-        <v>119</v>
-      </c>
-      <c r="G1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I1" t="s">
-        <v>124</v>
-      </c>
-      <c r="J1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I2" t="s">
-        <v>125</v>
-      </c>
-      <c r="J2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E4" t="s">
         <v>117</v>
       </c>
       <c r="F4">
         <v>1000</v>
       </c>
+      <c r="G4">
+        <v>50</v>
+      </c>
       <c r="H4">
-        <v>50</v>
-      </c>
-      <c r="J4">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -4776,14 +4717,14 @@
       <c r="F5">
         <v>3000</v>
       </c>
+      <c r="G5">
+        <v>80</v>
+      </c>
       <c r="H5">
-        <v>80</v>
-      </c>
-      <c r="J5">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
@@ -4802,10 +4743,10 @@
       <c r="F6">
         <v>5000</v>
       </c>
+      <c r="G6">
+        <v>100</v>
+      </c>
       <c r="H6">
-        <v>100</v>
-      </c>
-      <c r="J6">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update rules for Copilot assistant
Revised the system prompt to clarify Copilot's behavior, including response limitations, content policies, and developer-focused guidance. Ensured consistent branding and updated instructions for handling technical and non-technical queries.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KSSStudy\Projects\TangTang\Assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50ABDDA4-B70F-44F2-A687-3DF6E0D7CD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E3A993-A40A-4080-BE02-187FD84D97B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="8" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="3" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Player" sheetId="6" r:id="rId1"/>

</xml_diff>

<commit_message>
Add new feature to user profile page
Implemented additional functionality on the user profile page, including support for editing user details and updating the profile picture. Refactored related components for better maintainability.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E3A993-A40A-4080-BE02-187FD84D97B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910181EB-962F-46E4-A9DC-32FFCC619F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="3" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Player" sheetId="6" r:id="rId1"/>
     <sheet name="Hero" sheetId="10" r:id="rId2"/>
     <sheet name="HeroAcitveSkill" sheetId="16" r:id="rId3"/>
-    <sheet name="HeroPassiveSkill" sheetId="8" r:id="rId4"/>
+    <sheet name="HeroPassiveSkill" sheetId="17" r:id="rId4"/>
     <sheet name="HeroTranscendSkill" sheetId="9" r:id="rId5"/>
     <sheet name="NomalEnemy" sheetId="3" r:id="rId6"/>
     <sheet name="EliteEnemy" sheetId="13" r:id="rId7"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="238">
   <si>
     <t>Index</t>
   </si>
@@ -205,21 +205,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>공격력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>이동속도</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>아이템 획득 범위</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroActiveSkill_tigerPunch</t>
-  </si>
-  <si>
     <t>_heroActiveSkill_dragonBall</t>
   </si>
   <si>
@@ -229,668 +218,652 @@
     <t>_heroActiveSkill_electricField</t>
   </si>
   <si>
-    <t>_heroPassiveSkill_IronHelmet</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroPassiveSkill_AnalogClock</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroPassiveSkill_ChargePlug</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroPassiveSkill_WingShoes</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>_heroTranscendSkill_tigerPunch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroTranscendSkill_dragonBall</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroTranscendSkill_spinBlade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroTranscendSkill_electricField</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>뜨거운 주먹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>찾았다 xxx볼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅의 양쪽으로 주먹이 나왔다들어가며 적을 공격</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅으로부터 적을관통하며 직선으로 날아가는 공을 발사, 피격된 적 이동속도 1초간 0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅을 중심으로 영구히 회전하며 적을 공격</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반</t>
+  </si>
+  <si>
+    <t>정예</t>
+  </si>
+  <si>
+    <t>닭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>쥐</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>곰</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑우</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>다크바니</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_chicken</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_mouse</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_bear</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_blackCow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_darkBunny</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>죽음의 연꽃</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>료이키 텐카이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>타입</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>속성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Element</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Fire</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Water</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_chickenKing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>꼬꼬킹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ground</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wind</t>
+  </si>
+  <si>
+    <t>Wind</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dark</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정예</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기본체력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BaseMaxHp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기본공격력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BaseDamage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>등장하는 보스 적</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Normal Enemy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Elite Enemy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Boss Enemy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_snake</t>
+  </si>
+  <si>
+    <t>뱀</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>_enemy_crow</t>
+  </si>
+  <si>
+    <t>까마귀</t>
+  </si>
+  <si>
+    <t>_enemy_boar</t>
+  </si>
+  <si>
+    <t>멧돼지</t>
+  </si>
+  <si>
+    <t>_enemy_frog</t>
+  </si>
+  <si>
+    <t>개구리</t>
+  </si>
+  <si>
+    <t>_enemy_scorpion</t>
+  </si>
+  <si>
+    <t>전갈</t>
+  </si>
+  <si>
+    <t>_enemy_wolf</t>
+  </si>
+  <si>
+    <t>늑대</t>
+  </si>
+  <si>
+    <t>_enemy_crocodile</t>
+  </si>
+  <si>
+    <t>악어</t>
+  </si>
+  <si>
+    <t>_enemy_golem</t>
+  </si>
+  <si>
+    <t>골렘</t>
+  </si>
+  <si>
+    <t>골드</t>
+  </si>
+  <si>
+    <t>영웅 경험치</t>
+  </si>
+  <si>
+    <t>자석</t>
+  </si>
+  <si>
+    <t>공격력 업</t>
+  </si>
+  <si>
+    <t>체력 회복</t>
+  </si>
+  <si>
+    <t>폭탄</t>
+  </si>
+  <si>
+    <t>보물상자</t>
+  </si>
+  <si>
+    <t>당근</t>
+  </si>
+  <si>
+    <t>_dropItem_gold</t>
+  </si>
+  <si>
+    <t>_dropItem_carrot</t>
+  </si>
+  <si>
+    <t>_dropItem_magnet</t>
+  </si>
+  <si>
+    <t>_dropItem_atkUp</t>
+  </si>
+  <si>
+    <t>_dropItem_bomb</t>
+  </si>
+  <si>
+    <t>피스풀 평원</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>다크 심장부</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노이지 숲</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1,2,3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3,4,5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5,6,7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1,2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2,3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스폰되는 일반 적</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스폰되는 정예 적</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정예 적 스폰시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Elite Enemy SpawnTime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>60n</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스 적 스폰 시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Boss Enemy SpawnTime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_stage_Story1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_stage_Story2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_stage_Story3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_stage_Survive1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>존재하며 버티기</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1,2,3,4,5,6,7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>승리조건</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Victory Condition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>승리조건 설명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vic Description</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스처치 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제한시간 생존</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제한시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TimeLimit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>LocalizationKey</t>
+  </si>
+  <si>
+    <t>CoolTime</t>
+  </si>
+  <si>
+    <t>영웅으로부터 주먹이 나왔다들어가며 적을 공격</t>
+  </si>
+  <si>
+    <t>영웅으로부터 적을 관통하며 직선으로 날아가는 공을 발사</t>
+  </si>
+  <si>
+    <t>영웅을 중심으로 회전하며 적을 공격</t>
+  </si>
+  <si>
+    <t>전기장</t>
+  </si>
+  <si>
+    <t>영웅을 중심으로 원을 생성하여 범위 안의 적을 공격</t>
+  </si>
+  <si>
+    <t>총총총</t>
+  </si>
+  <si>
+    <t>영웅을 중심으로 총알을 생성하여 가장 가까운 적을 공격</t>
+  </si>
+  <si>
+    <t>BulletSpeed</t>
+  </si>
+  <si>
+    <t>ShootingRange</t>
+  </si>
+  <si>
+    <t>BulletCount</t>
+  </si>
+  <si>
+    <t>BulletDuration</t>
+  </si>
+  <si>
+    <t>FireDelay</t>
+  </si>
+  <si>
+    <t>AttackCount</t>
+  </si>
+  <si>
+    <t>BulletRange</t>
+  </si>
+  <si>
+    <t>RotSpeed</t>
+  </si>
+  <si>
+    <t>DamageDelay</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>_dropItem_heroExp</t>
+  </si>
+  <si>
+    <t>_dropItem_hpPotion</t>
+  </si>
+  <si>
+    <t>KillAllEnemies</t>
+  </si>
+  <si>
+    <t>_dropItem_treasureBox</t>
+  </si>
+  <si>
+    <t>DropTreasureBox</t>
+  </si>
+  <si>
+    <t>AttractAllItems</t>
+  </si>
+  <si>
+    <t>DropCondition</t>
+  </si>
+  <si>
+    <t>일반 적 처치시, 확률에따라</t>
+  </si>
+  <si>
+    <t>플레이어가 골드를 5만큼 획득합니다. (장비 강화 등에 사용)</t>
+  </si>
+  <si>
+    <t>정예 적 처치시, 반드시 1개를 드롭보스 처치시, 반드시 3개를 드롭</t>
+  </si>
+  <si>
+    <t>플레이어가 당근 1개를 획득합니다. (장비 뽑기 등에 사용)</t>
+  </si>
+  <si>
+    <t>영웅이 경험치를 5만큼 획득합니다. (스킬 선택/강화에 사용)</t>
+  </si>
+  <si>
+    <t>맵 전체에 있는 모든 아이템을 끌어당깁니다.</t>
+  </si>
+  <si>
+    <t>10초간 공격력이 20%만큼 증가합니다. (일시적 버프)</t>
+  </si>
+  <si>
+    <t>일반 적 처치시, 확률에따라보스 처치시, 반드시 1개를 드롭</t>
+  </si>
+  <si>
+    <t>영웅의 체력이 20%만큼 회복됩니다.</t>
+  </si>
+  <si>
+    <t>맵에 있는 일반/정예 적 전부를 즉시 처치합니다. (보스 제외)</t>
+  </si>
+  <si>
+    <t>보스 처치시, 반드시 1개를 드롭</t>
+  </si>
+  <si>
+    <t>무작위 공격/패시브 스킬의 레벨이 1 증가합니다. 이 효과는 random(1~5)회 반복됩니다.</t>
+  </si>
+  <si>
+    <t>GoldAmount</t>
+  </si>
+  <si>
+    <t>CarrotAmount</t>
+  </si>
+  <si>
+    <t>ExpAmount</t>
+  </si>
+  <si>
+    <t>HpHealPercent</t>
+  </si>
+  <si>
+    <t>AtkBuffPercent</t>
+  </si>
+  <si>
+    <t>BuffDurationSec</t>
+  </si>
+  <si>
+    <t>SpecialEffectKey</t>
+  </si>
+  <si>
+    <t>DropChance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BaseMaxHp</t>
+  </si>
+  <si>
+    <t>HpGrowthRate</t>
+  </si>
+  <si>
+    <t>BaseDamage</t>
+  </si>
+  <si>
+    <t>DamageGrowthRate</t>
+  </si>
+  <si>
+    <t>BaseMoveSpeed</t>
+  </si>
+  <si>
+    <t>MoveSpeedGrowthRate</t>
+  </si>
+  <si>
+    <t>BaseItemGetRange</t>
+  </si>
+  <si>
+    <t>ItemGetRangeGrowthRate</t>
+  </si>
+  <si>
+    <t>BaseExpToLevelUp</t>
+  </si>
+  <si>
+    <t>ExpRequiredGrowthRate</t>
+  </si>
+  <si>
+    <t>MaxLevel</t>
+  </si>
+  <si>
+    <t>BaseExpGainRate</t>
+  </si>
+  <si>
+    <t>_hero_bunnyTiger</t>
+  </si>
+  <si>
+    <t>바니호걸</t>
+  </si>
+  <si>
+    <t>_hero_bunnyDragon</t>
+  </si>
+  <si>
+    <t>바니에용</t>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroActiveSkill_hogirlPunch</t>
+  </si>
+  <si>
+    <t>_heroActiveSkill_gun</t>
+  </si>
+  <si>
+    <t>EffectType</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
   <si>
     <t>아날로그시계</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅의 스테이지 시작 시 드롭 확률을 기준으로 증가</t>
   </si>
   <si>
     <t>철제투구</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxHp</t>
+  </si>
+  <si>
+    <t>영웅의 스테이지 시작 시 최대 체력을 기준으로 증가</t>
   </si>
   <si>
     <t>충전플러그</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>영웅의 스테이지 시작 시 공격력을 기준으로 증가</t>
   </si>
   <si>
     <t>윙슈즈</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>증가시킬 스탯</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TargetStat</t>
-  </si>
-  <si>
-    <t>Increase</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스탯 증가량</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroTranscendSkill_tigerPunch</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroTranscendSkill_dragonBall</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroTranscendSkill_spinBlade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_heroTranscendSkill_electricField</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>뜨거운 주먹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>찾았다 xxx볼</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅의 양쪽으로 주먹이 나왔다들어가며 적을 공격</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅으로부터 적을관통하며 직선으로 날아가는 공을 발사, 피격된 적 이동속도 1초간 0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅을 중심으로 영구히 회전하며 적을 공격</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>일반</t>
-  </si>
-  <si>
-    <t>정예</t>
-  </si>
-  <si>
-    <t>최대 체력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스킬 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Description</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>닭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>쥐</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>곰</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑우</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>다크바니</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_chicken</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_mouse</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_bear</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_blackCow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_darkBunny</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>죽음의 연꽃</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>료이키 텐카이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>타입</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>속성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Element</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Fire</t>
-  </si>
-  <si>
-    <t>Fire</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Water</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_chickenKing</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>꼬꼬킹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ground</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Wind</t>
-  </si>
-  <si>
-    <t>Wind</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dark</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>일반</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보스</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>정예</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>기본체력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BaseMaxHp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>기본공격력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BaseDamage</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>영웅의 스테이지 시작 시 이동속도를 기준으로 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅의 스테이지 시작 시 공격력을 기준으로 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅의 스테이지 시작 시 최대 체력을 기준으로 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅의 스테이지 시작 시 드롭 확률을 기준으로 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>등장하는 보스 적</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Normal Enemy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Elite Enemy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Boss Enemy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_snake</t>
-  </si>
-  <si>
-    <t>뱀</t>
-  </si>
-  <si>
-    <t>Earth</t>
-  </si>
-  <si>
-    <t>_enemy_crow</t>
-  </si>
-  <si>
-    <t>까마귀</t>
-  </si>
-  <si>
-    <t>_enemy_boar</t>
-  </si>
-  <si>
-    <t>멧돼지</t>
-  </si>
-  <si>
-    <t>_enemy_frog</t>
-  </si>
-  <si>
-    <t>개구리</t>
-  </si>
-  <si>
-    <t>_enemy_scorpion</t>
-  </si>
-  <si>
-    <t>전갈</t>
-  </si>
-  <si>
-    <t>_enemy_wolf</t>
-  </si>
-  <si>
-    <t>늑대</t>
-  </si>
-  <si>
-    <t>_enemy_crocodile</t>
-  </si>
-  <si>
-    <t>악어</t>
-  </si>
-  <si>
-    <t>_enemy_golem</t>
-  </si>
-  <si>
-    <t>골렘</t>
-  </si>
-  <si>
-    <t>골드</t>
-  </si>
-  <si>
-    <t>영웅 경험치</t>
-  </si>
-  <si>
-    <t>자석</t>
-  </si>
-  <si>
-    <t>공격력 업</t>
-  </si>
-  <si>
-    <t>체력 회복</t>
-  </si>
-  <si>
-    <t>폭탄</t>
-  </si>
-  <si>
-    <t>보물상자</t>
-  </si>
-  <si>
-    <t>당근</t>
-  </si>
-  <si>
-    <t>_dropItem_gold</t>
-  </si>
-  <si>
-    <t>_dropItem_carrot</t>
-  </si>
-  <si>
-    <t>_dropItem_magnet</t>
-  </si>
-  <si>
-    <t>_dropItem_atkUp</t>
-  </si>
-  <si>
-    <t>_dropItem_bomb</t>
-  </si>
-  <si>
-    <t>피스풀 평원</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>다크 심장부</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>노이지 숲</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1,2,3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3,4,5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>5,6,7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1,2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2,3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스폰되는 일반 적</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스폰되는 정예 적</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>정예 적 스폰시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Elite Enemy SpawnTime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>60n</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보스 적 스폰 시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Boss Enemy SpawnTime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_stage_Story1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_stage_Story2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_stage_Story3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_stage_Survive1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>존재하며 버티기</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1,2,3,4,5,6,7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>승리조건</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Victory Condition</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>승리조건 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vic Description</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보스처치 완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>제한시간 생존</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>제한시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TimeLimit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>LocalizationKey</t>
-  </si>
-  <si>
-    <t>CoolTime</t>
-  </si>
-  <si>
-    <t>영웅으로부터 주먹이 나왔다들어가며 적을 공격</t>
-  </si>
-  <si>
-    <t>영웅으로부터 적을 관통하며 직선으로 날아가는 공을 발사</t>
-  </si>
-  <si>
-    <t>영웅을 중심으로 회전하며 적을 공격</t>
-  </si>
-  <si>
-    <t>전기장</t>
-  </si>
-  <si>
-    <t>영웅을 중심으로 원을 생성하여 범위 안의 적을 공격</t>
-  </si>
-  <si>
-    <t>_heroActiveSkill_Gun</t>
-  </si>
-  <si>
-    <t>총총총</t>
-  </si>
-  <si>
-    <t>영웅을 중심으로 총알을 생성하여 가장 가까운 적을 공격</t>
-  </si>
-  <si>
-    <t>BulletSpeed</t>
-  </si>
-  <si>
-    <t>ShootingRange</t>
-  </si>
-  <si>
-    <t>BulletCount</t>
-  </si>
-  <si>
-    <t>BulletDuration</t>
-  </si>
-  <si>
-    <t>FireDelay</t>
-  </si>
-  <si>
-    <t>AttackCount</t>
-  </si>
-  <si>
-    <t>BulletRange</t>
-  </si>
-  <si>
-    <t>RotSpeed</t>
-  </si>
-  <si>
-    <t>DamageDelay</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>_dropItem_heroExp</t>
-  </si>
-  <si>
-    <t>_dropItem_hpPotion</t>
-  </si>
-  <si>
-    <t>KillAllEnemies</t>
-  </si>
-  <si>
-    <t>_dropItem_treasureBox</t>
-  </si>
-  <si>
-    <t>DropTreasureBox</t>
-  </si>
-  <si>
-    <t>AttractAllItems</t>
-  </si>
-  <si>
-    <t>DropCondition</t>
-  </si>
-  <si>
-    <t>일반 적 처치시, 확률에따라</t>
-  </si>
-  <si>
-    <t>플레이어가 골드를 5만큼 획득합니다. (장비 강화 등에 사용)</t>
-  </si>
-  <si>
-    <t>정예 적 처치시, 반드시 1개를 드롭보스 처치시, 반드시 3개를 드롭</t>
-  </si>
-  <si>
-    <t>플레이어가 당근 1개를 획득합니다. (장비 뽑기 등에 사용)</t>
-  </si>
-  <si>
-    <t>영웅이 경험치를 5만큼 획득합니다. (스킬 선택/강화에 사용)</t>
-  </si>
-  <si>
-    <t>맵 전체에 있는 모든 아이템을 끌어당깁니다.</t>
-  </si>
-  <si>
-    <t>10초간 공격력이 20%만큼 증가합니다. (일시적 버프)</t>
-  </si>
-  <si>
-    <t>일반 적 처치시, 확률에따라보스 처치시, 반드시 1개를 드롭</t>
-  </si>
-  <si>
-    <t>영웅의 체력이 20%만큼 회복됩니다.</t>
-  </si>
-  <si>
-    <t>맵에 있는 일반/정예 적 전부를 즉시 처치합니다. (보스 제외)</t>
-  </si>
-  <si>
-    <t>보스 처치시, 반드시 1개를 드롭</t>
-  </si>
-  <si>
-    <t>무작위 공격/패시브 스킬의 레벨이 1 증가합니다. 이 효과는 random(1~5)회 반복됩니다.</t>
-  </si>
-  <si>
-    <t>GoldAmount</t>
-  </si>
-  <si>
-    <t>CarrotAmount</t>
-  </si>
-  <si>
-    <t>ExpAmount</t>
-  </si>
-  <si>
-    <t>HpHealPercent</t>
-  </si>
-  <si>
-    <t>AtkBuffPercent</t>
-  </si>
-  <si>
-    <t>BuffDurationSec</t>
-  </si>
-  <si>
-    <t>SpecialEffectKey</t>
-  </si>
-  <si>
-    <t>DropChance</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BaseMaxHp</t>
-  </si>
-  <si>
-    <t>HpGrowthRate</t>
-  </si>
-  <si>
-    <t>BaseDamage</t>
-  </si>
-  <si>
-    <t>DamageGrowthRate</t>
-  </si>
-  <si>
-    <t>BaseMoveSpeed</t>
-  </si>
-  <si>
-    <t>MoveSpeedGrowthRate</t>
-  </si>
-  <si>
-    <t>BaseItemGetRange</t>
-  </si>
-  <si>
-    <t>ItemGetRangeGrowthRate</t>
-  </si>
-  <si>
-    <t>BaseExpToLevelUp</t>
-  </si>
-  <si>
-    <t>ExpRequiredGrowthRate</t>
-  </si>
-  <si>
-    <t>MaxLevel</t>
-  </si>
-  <si>
-    <t>BaseExpGainRate</t>
-  </si>
-  <si>
-    <t>_hero_bunnyTiger</t>
-  </si>
-  <si>
-    <t>바니호걸</t>
-  </si>
-  <si>
-    <t>_hero_bunnyDragon</t>
-  </si>
-  <si>
-    <t>바니에용</t>
-  </si>
-  <si>
-    <t>Name</t>
+  </si>
+  <si>
+    <t>ItemGetRange</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroPassiveSkill_analogClock</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroPassiveSkill_ironHelmet</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroPassiveSkill_chargePlug</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_heroPassiveSkill_wingShoes</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -940,7 +913,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -963,24 +936,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -988,38 +950,20 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1381,28 +1325,28 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
-        <v>156</v>
+        <v>134</v>
       </c>
       <c r="E1" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="F1" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="G1" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="H1" t="s">
-        <v>161</v>
+        <v>139</v>
       </c>
       <c r="I1" t="s">
-        <v>169</v>
+        <v>147</v>
       </c>
       <c r="J1" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="K1" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1416,28 +1360,28 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="F2" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="G2" t="s">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="H2" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="I2" t="s">
-        <v>170</v>
+        <v>148</v>
       </c>
       <c r="J2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="K2" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -1480,19 +1424,19 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="E4" t="s">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="F4" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -1504,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -1512,19 +1456,19 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>142</v>
       </c>
       <c r="C5" t="s">
-        <v>150</v>
+        <v>128</v>
       </c>
       <c r="D5" t="s">
-        <v>152</v>
+        <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="F5" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="G5">
         <v>2</v>
@@ -1536,7 +1480,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -1544,19 +1488,19 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="E6" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="F6" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -1568,7 +1512,7 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -1576,25 +1520,25 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>144</v>
       </c>
       <c r="C7" t="s">
-        <v>167</v>
+        <v>145</v>
       </c>
       <c r="D7" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="F7" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="I7" t="b">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="K7">
         <v>600</v>
@@ -1627,49 +1571,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
       <c r="B1" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>174</v>
       </c>
       <c r="D1" t="s">
-        <v>225</v>
+        <v>202</v>
       </c>
       <c r="E1" t="s">
-        <v>226</v>
+        <v>203</v>
       </c>
       <c r="F1" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="G1" t="s">
-        <v>228</v>
+        <v>205</v>
       </c>
       <c r="H1" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="I1" t="s">
-        <v>230</v>
+        <v>207</v>
       </c>
       <c r="J1" t="s">
-        <v>231</v>
+        <v>208</v>
       </c>
       <c r="K1" t="s">
-        <v>232</v>
+        <v>209</v>
       </c>
       <c r="L1" t="s">
-        <v>233</v>
+        <v>210</v>
       </c>
       <c r="M1" t="s">
-        <v>234</v>
+        <v>211</v>
       </c>
       <c r="N1" t="s">
-        <v>235</v>
+        <v>212</v>
       </c>
       <c r="O1" t="s">
-        <v>236</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -1677,10 +1621,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>237</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>238</v>
+        <v>215</v>
       </c>
       <c r="D2">
         <v>200</v>
@@ -1724,10 +1668,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>239</v>
+        <v>216</v>
       </c>
       <c r="C3" t="s">
-        <v>240</v>
+        <v>217</v>
       </c>
       <c r="D3">
         <v>200</v>
@@ -1779,10 +1723,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
       <c r="B1" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
@@ -1794,34 +1738,34 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="G1" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="H1" t="s">
-        <v>190</v>
+        <v>167</v>
       </c>
       <c r="I1" t="s">
-        <v>191</v>
+        <v>168</v>
       </c>
       <c r="J1" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="K1" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="L1" t="s">
-        <v>193</v>
+        <v>170</v>
       </c>
       <c r="M1" t="s">
-        <v>194</v>
+        <v>171</v>
       </c>
       <c r="N1" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="O1" t="s">
-        <v>196</v>
+        <v>173</v>
       </c>
       <c r="P1" t="s">
         <v>15</v>
@@ -1838,7 +1782,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>219</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -1859,10 +1803,10 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1871,7 +1815,7 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1886,7 +1830,7 @@
         <v>23</v>
       </c>
       <c r="R2" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -1894,7 +1838,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>219</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -1915,7 +1859,7 @@
         <v>1</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1927,7 +1871,7 @@
         <v>1</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -1942,7 +1886,7 @@
         <v>23</v>
       </c>
       <c r="R3" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -1950,7 +1894,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>219</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -1971,7 +1915,7 @@
         <v>2</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>2</v>
@@ -1983,7 +1927,7 @@
         <v>1</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -1998,7 +1942,7 @@
         <v>23</v>
       </c>
       <c r="R4" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -2006,7 +1950,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>219</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -2027,7 +1971,7 @@
         <v>2</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>2</v>
@@ -2039,7 +1983,7 @@
         <v>1</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -2054,7 +1998,7 @@
         <v>23</v>
       </c>
       <c r="R5" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
@@ -2062,7 +2006,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>219</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -2083,7 +2027,7 @@
         <v>3</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>2</v>
@@ -2095,7 +2039,7 @@
         <v>1</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -2110,7 +2054,7 @@
         <v>23</v>
       </c>
       <c r="R6" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
@@ -2118,7 +2062,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>
@@ -2130,16 +2074,16 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
         <v>2</v>
@@ -2148,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="M7">
         <v>5</v>
@@ -2166,7 +2110,7 @@
         <v>23</v>
       </c>
       <c r="R7" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -2174,7 +2118,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -2186,7 +2130,7 @@
         <v>1.2</v>
       </c>
       <c r="F8">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -2222,7 +2166,7 @@
         <v>23</v>
       </c>
       <c r="R8" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
@@ -2230,7 +2174,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -2242,7 +2186,7 @@
         <v>1.4</v>
       </c>
       <c r="F9">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -2278,7 +2222,7 @@
         <v>23</v>
       </c>
       <c r="R9" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
@@ -2286,7 +2230,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
         <v>24</v>
@@ -2298,7 +2242,7 @@
         <v>1.6</v>
       </c>
       <c r="F10">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -2334,7 +2278,7 @@
         <v>23</v>
       </c>
       <c r="R10" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -2342,7 +2286,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
@@ -2354,7 +2298,7 @@
         <v>1.8</v>
       </c>
       <c r="F11">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -2390,7 +2334,7 @@
         <v>23</v>
       </c>
       <c r="R11" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
@@ -2398,7 +2342,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C12" t="s">
         <v>25</v>
@@ -2410,7 +2354,7 @@
         <v>0.7</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -2422,7 +2366,7 @@
         <v>3</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12">
         <v>0</v>
@@ -2446,7 +2390,7 @@
         <v>23</v>
       </c>
       <c r="R12" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -2454,7 +2398,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
         <v>25</v>
@@ -2466,7 +2410,7 @@
         <v>0.9</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G13">
         <v>2</v>
@@ -2478,7 +2422,7 @@
         <v>3.25</v>
       </c>
       <c r="J13">
-        <v>5</v>
+        <v>2.75</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -2502,7 +2446,7 @@
         <v>23</v>
       </c>
       <c r="R13" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
@@ -2510,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
         <v>25</v>
@@ -2522,7 +2466,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G14">
         <v>2</v>
@@ -2534,7 +2478,7 @@
         <v>3.5</v>
       </c>
       <c r="J14">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -2558,7 +2502,7 @@
         <v>23</v>
       </c>
       <c r="R14" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
@@ -2566,7 +2510,7 @@
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
         <v>25</v>
@@ -2578,7 +2522,7 @@
         <v>1.3</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G15">
         <v>2</v>
@@ -2590,7 +2534,7 @@
         <v>3.75</v>
       </c>
       <c r="J15">
-        <v>5</v>
+        <v>2.25</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -2614,7 +2558,7 @@
         <v>23</v>
       </c>
       <c r="R15" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
@@ -2622,7 +2566,7 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
         <v>25</v>
@@ -2634,7 +2578,7 @@
         <v>1.5</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="G16">
         <v>2</v>
@@ -2646,7 +2590,7 @@
         <v>4</v>
       </c>
       <c r="J16">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K16">
         <v>0</v>
@@ -2670,7 +2614,7 @@
         <v>23</v>
       </c>
       <c r="R16" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -2678,10 +2622,10 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2705,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17">
         <v>1</v>
@@ -2726,7 +2670,7 @@
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -2734,10 +2678,10 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2761,7 +2705,7 @@
         <v>0</v>
       </c>
       <c r="K18">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="L18">
         <v>1</v>
@@ -2782,7 +2726,7 @@
         <v>23</v>
       </c>
       <c r="R18" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -2790,10 +2734,10 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -2817,7 +2761,7 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L19">
         <v>1</v>
@@ -2838,7 +2782,7 @@
         <v>23</v>
       </c>
       <c r="R19" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
@@ -2846,10 +2790,10 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C20" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D20">
         <v>4</v>
@@ -2873,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="K20">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="L20">
         <v>1</v>
@@ -2894,7 +2838,7 @@
         <v>23</v>
       </c>
       <c r="R20" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
@@ -2902,10 +2846,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="D21">
         <v>5</v>
@@ -2929,10 +2873,10 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21">
         <v>3</v>
@@ -2950,7 +2894,7 @@
         <v>23</v>
       </c>
       <c r="R21" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
@@ -2958,10 +2902,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C22" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2970,22 +2914,22 @@
         <v>1</v>
       </c>
       <c r="F22">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <v>1</v>
       </c>
       <c r="K22">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -3006,7 +2950,7 @@
         <v>23</v>
       </c>
       <c r="R22" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
@@ -3014,10 +2958,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C23" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D23">
         <v>2</v>
@@ -3026,22 +2970,22 @@
         <v>1.2</v>
       </c>
       <c r="F23">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L23">
         <v>1</v>
@@ -3062,7 +3006,7 @@
         <v>23</v>
       </c>
       <c r="R23" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
@@ -3070,10 +3014,10 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C24" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -3082,22 +3026,22 @@
         <v>1.5</v>
       </c>
       <c r="F24">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H24">
         <v>3</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="K24">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L24">
         <v>1</v>
@@ -3118,7 +3062,7 @@
         <v>23</v>
       </c>
       <c r="R24" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
@@ -3126,10 +3070,10 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C25" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -3138,22 +3082,22 @@
         <v>1.7</v>
       </c>
       <c r="F25">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="L25">
         <v>1</v>
@@ -3174,7 +3118,7 @@
         <v>23</v>
       </c>
       <c r="R25" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
@@ -3182,10 +3126,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C26" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -3194,22 +3138,22 @@
         <v>2</v>
       </c>
       <c r="F26">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="K26">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="L26">
         <v>1</v>
@@ -3230,7 +3174,7 @@
         <v>23</v>
       </c>
       <c r="R26" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3240,549 +3184,506 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D47192C-7E49-4B79-BE34-99145BC381BF}">
-  <dimension ref="A1:G23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83F5C8F2-E7C1-447E-84A4-DCD685841AE4}">
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="3.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>62</v>
+      <c r="A1" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>222</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D2" s="7">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="7">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" s="7">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="7">
+        <v>3</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D5" s="7">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" s="7">
         <v>5</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E6" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F6" s="7">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D7" s="7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
+        <v>2</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" s="7">
+        <v>2</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
+        <v>2</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F9" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="7">
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D10" s="7">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="8">
-        <v>1</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" s="8">
+      <c r="E10" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F10" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="7">
+        <v>2</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11" s="7">
+        <v>5</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="7">
+        <v>3</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F12" s="7">
         <v>0.2</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
-        <v>1</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" s="8">
-        <v>2</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" s="8">
+      <c r="G12" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="7">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F13" s="7">
         <v>0.4</v>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="8">
-        <v>3</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6" s="8">
+      <c r="G13" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="7">
+        <v>3</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="7">
+        <v>3</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F14" s="7">
         <v>0.6</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
-        <v>1</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="G14" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="7">
+        <v>3</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="7">
         <v>4</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="8">
+      <c r="E15" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F15" s="7">
         <v>0.8</v>
       </c>
-      <c r="G7" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
-        <v>1</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="8">
+      <c r="G15" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="7">
+        <v>3</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D16" s="7">
         <v>5</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="8">
-        <v>1</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
-        <v>2</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" s="8">
-        <v>1</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F9" s="8">
+      <c r="E16" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>4</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D17" s="7">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="7">
         <v>0.2</v>
       </c>
-      <c r="G9" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
-        <v>2</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="8">
-        <v>2</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10" s="8">
+      <c r="G17" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="7">
+        <v>4</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D18" s="7">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="7">
         <v>0.4</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
-        <v>2</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="8">
-        <v>3</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" s="8">
+      <c r="G18" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="7">
+        <v>4</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D19" s="7">
+        <v>3</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="7">
         <v>0.6</v>
       </c>
-      <c r="G11" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
-        <v>2</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="8">
+      <c r="G19" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="7">
         <v>4</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F12" s="8">
+      <c r="B20" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D20" s="7">
+        <v>4</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="7">
         <v>0.8</v>
       </c>
-      <c r="G12" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="8">
-        <v>2</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="8">
+      <c r="G20" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="7">
+        <v>4</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D21" s="7">
         <v>5</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="8">
-        <v>1</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
-        <v>3</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="8">
-        <v>1</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="8">
-        <v>3</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="8">
-        <v>2</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F15" s="8">
-        <v>0.4</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
-        <v>3</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="8">
-        <v>3</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F16" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="8">
-        <v>3</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="8">
-        <v>4</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="8">
-        <v>0.8</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="8">
-        <v>3</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="8">
-        <v>5</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F18" s="8">
-        <v>1</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="8">
-        <v>4</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="8">
-        <v>1</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="8">
-        <v>4</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="8">
-        <v>2</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20" s="8">
-        <v>0.4</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="8">
-        <v>4</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="8">
-        <v>3</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="8">
-        <v>4</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="8">
-        <v>4</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="8">
-        <v>0.8</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="8">
-        <v>4</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="8">
-        <v>5</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="8">
-        <v>1</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>110</v>
+      <c r="E21" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="7">
+        <v>1</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3807,143 +3708,143 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3952,10 +3853,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -3981,7 +3882,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -3989,10 +3890,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -4020,7 +3921,7 @@
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -4028,10 +3929,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -4059,7 +3960,7 @@
         <v>90</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -4067,10 +3968,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -4125,19 +4026,19 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
       <c r="H1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -4151,16 +4052,16 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" t="s">
         <v>91</v>
-      </c>
-      <c r="E2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G2" t="s">
-        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -4197,16 +4098,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E4" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <v>50</v>
@@ -4223,16 +4124,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F5">
         <v>30</v>
@@ -4249,16 +4150,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1">
         <v>45</v>
@@ -4275,16 +4176,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="F7" s="1">
         <v>35</v>
@@ -4301,16 +4202,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F8" s="1">
         <v>60</v>
@@ -4327,16 +4228,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F9" s="1">
         <v>40</v>
@@ -4353,16 +4254,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F10" s="1">
         <v>55</v>
@@ -4406,19 +4307,19 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
       <c r="H1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -4432,16 +4333,16 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" t="s">
         <v>91</v>
-      </c>
-      <c r="E2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G2" t="s">
-        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -4478,16 +4379,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="F4">
         <v>200</v>
@@ -4504,16 +4405,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="F5" s="1">
         <v>180</v>
@@ -4530,16 +4431,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="F6" s="1">
         <v>220</v>
@@ -4556,16 +4457,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="F7" s="1">
         <v>300</v>
@@ -4609,19 +4510,19 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G1" t="s">
-        <v>108</v>
-      </c>
       <c r="H1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -4635,16 +4536,16 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" t="s">
         <v>91</v>
-      </c>
-      <c r="E2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G2" t="s">
-        <v>109</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -4681,16 +4582,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E4" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="F4">
         <v>1000</v>
@@ -4707,16 +4608,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="F5">
         <v>3000</v>
@@ -4733,16 +4634,16 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" t="s">
         <v>86</v>
-      </c>
-      <c r="C6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" t="s">
-        <v>104</v>
       </c>
       <c r="F6">
         <v>5000</v>
@@ -4780,43 +4681,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="E1" s="13" t="s">
+      <c r="A1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="J1" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="L1" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="M1" s="13" t="s">
+      <c r="D1" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4825,10 +4726,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="D2" s="1">
         <v>5</v>
@@ -4840,13 +4741,13 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L2" s="1">
         <v>100</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4854,10 +4755,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1">
@@ -4869,11 +4770,11 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1" t="s">
-        <v>207</v>
+        <v>184</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
-        <v>208</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -4881,10 +4782,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>175</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -4896,13 +4797,13 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L4" s="1">
         <v>100</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -4910,10 +4811,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>137</v>
+        <v>115</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4922,16 +4823,16 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>203</v>
+        <v>180</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L5" s="1">
         <v>1</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>210</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -4939,10 +4840,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -4956,13 +4857,13 @@
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L6" s="1">
         <v>1</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>211</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4970,10 +4871,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>199</v>
+        <v>176</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -4985,13 +4886,13 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>212</v>
+        <v>189</v>
       </c>
       <c r="L7" s="1">
         <v>1</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>213</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -4999,10 +4900,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -5011,16 +4912,16 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L8" s="1">
         <v>1</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>214</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -5028,10 +4929,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -5040,14 +4941,14 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>202</v>
+        <v>179</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>215</v>
+        <v>192</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -5061,16 +4962,16 @@
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>

</xml_diff>

<commit_message>
Refactor hero stats and implement object pooling
Introduced HeroModel, HeroStats, and Stat classes to refactor hero stat management. Updated Hero, ActiveSkill, and skill scripts to use the new stat system and events. Replaced direct bullet instantiation with object pooling for all hero skills and bullets, improving performance and resource management. Removed unused fields and updated data readers and ScriptableObjects to support new prefab and icon references. Added new prefabs and icons for passive skills.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910181EB-962F-46E4-A9DC-32FFCC619F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55664ADE-C9F1-412B-8272-A428D7305B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="3" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="8" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Player" sheetId="6" r:id="rId1"/>
@@ -713,9 +713,6 @@
     <t>10초간 공격력이 20%만큼 증가합니다. (일시적 버프)</t>
   </si>
   <si>
-    <t>일반 적 처치시, 확률에따라보스 처치시, 반드시 1개를 드롭</t>
-  </si>
-  <si>
     <t>영웅의 체력이 20%만큼 회복됩니다.</t>
   </si>
   <si>
@@ -864,6 +861,11 @@
   </si>
   <si>
     <t>_heroPassiveSkill_wingShoes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반 적 처치시, 확률에따라
+보스 처치시, 반드시 1개를 드롭</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1580,40 +1582,40 @@
         <v>174</v>
       </c>
       <c r="D1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" t="s">
         <v>202</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>203</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>204</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>205</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>206</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>207</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>208</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>209</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>210</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>211</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>212</v>
-      </c>
-      <c r="O1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -1621,10 +1623,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" t="s">
         <v>214</v>
-      </c>
-      <c r="C2" t="s">
-        <v>215</v>
       </c>
       <c r="D2">
         <v>200</v>
@@ -1668,10 +1670,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" t="s">
         <v>216</v>
-      </c>
-      <c r="C3" t="s">
-        <v>217</v>
       </c>
       <c r="D3">
         <v>200</v>
@@ -1782,7 +1784,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -1838,7 +1840,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -1894,7 +1896,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -1950,7 +1952,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -2006,7 +2008,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -2902,7 +2904,7 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C22" t="s">
         <v>163</v>
@@ -2958,7 +2960,7 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C23" t="s">
         <v>163</v>
@@ -3014,7 +3016,7 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C24" t="s">
         <v>163</v>
@@ -3070,7 +3072,7 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C25" t="s">
         <v>163</v>
@@ -3126,7 +3128,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C26" t="s">
         <v>163</v>
@@ -3211,10 +3213,10 @@
         <v>4</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>221</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>222</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>14</v>
@@ -3225,22 +3227,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D2" s="7">
         <v>1</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F2" s="7">
         <v>0.2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -3248,22 +3250,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="7">
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F3" s="7">
         <v>0.4</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3271,22 +3273,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D4" s="7">
         <v>3</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F4" s="7">
         <v>0.6</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3294,22 +3296,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D5" s="7">
         <v>4</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F5" s="7">
         <v>0.8</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3317,22 +3319,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D6" s="7">
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3340,22 +3342,22 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" s="7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="D7" s="7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="F7" s="7">
         <v>0.2</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3363,22 +3365,22 @@
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="7">
+        <v>2</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="D8" s="7">
-        <v>2</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="F8" s="7">
         <v>0.4</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3386,22 +3388,22 @@
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="D9" s="7">
-        <v>3</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="F9" s="7">
         <v>0.6</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3409,22 +3411,22 @@
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D10" s="7">
         <v>4</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F10" s="7">
         <v>0.8</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3432,22 +3434,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D11" s="7">
         <v>5</v>
       </c>
       <c r="E11" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="F11" s="7">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>226</v>
-      </c>
-      <c r="F11" s="7">
-        <v>1</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3455,22 +3457,22 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="D12" s="7">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="F12" s="7">
         <v>0.2</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -3478,22 +3480,22 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="D13" s="7">
-        <v>2</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="F13" s="7">
         <v>0.4</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -3501,22 +3503,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D14" s="7">
+        <v>3</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="D14" s="7">
-        <v>3</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="F14" s="7">
         <v>0.6</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -3524,22 +3526,22 @@
         <v>3</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D15" s="7">
         <v>4</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F15" s="7">
         <v>0.8</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -3547,22 +3549,22 @@
         <v>3</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D16" s="7">
         <v>5</v>
       </c>
       <c r="E16" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7" t="s">
         <v>229</v>
-      </c>
-      <c r="F16" s="7">
-        <v>1</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -3570,10 +3572,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D17" s="7">
         <v>1</v>
@@ -3585,7 +3587,7 @@
         <v>0.2</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -3593,10 +3595,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D18" s="7">
         <v>2</v>
@@ -3608,7 +3610,7 @@
         <v>0.4</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -3616,10 +3618,10 @@
         <v>4</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D19" s="7">
         <v>3</v>
@@ -3631,7 +3633,7 @@
         <v>0.6</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -3639,10 +3641,10 @@
         <v>4</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D20" s="7">
         <v>4</v>
@@ -3654,7 +3656,7 @@
         <v>0.8</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -3662,10 +3664,10 @@
         <v>4</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D21" s="7">
         <v>5</v>
@@ -3677,7 +3679,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -4481,6 +4483,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4688,34 +4691,34 @@
         <v>156</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>181</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>14</v>
@@ -4886,13 +4889,13 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="L7" s="1">
-        <v>1</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -4921,7 +4924,7 @@
         <v>1</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4944,11 +4947,11 @@
         <v>179</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Refactor enemy system and add elemental/rush mechanics
Refactored the enemy state system into separate classes, introduced elemental types and calculation logic, and added support for rush-type enemies with the IRushable interface and RushEnemy class. Updated Enemy, EnemyModel, and HeroModel to support elemental damage and new state transitions. Added HeroManager, new prefabs, and animator/controller assets for expanded enemy types. Cleaned up and extended data structures in EnemyStatData, and updated event and interface signatures for damage handling.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288534C8-4853-4ACE-9837-6C5489E85564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCE8DB2-E398-44C1-936D-AF271C1867AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="8" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="5" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Player" sheetId="6" r:id="rId1"/>
@@ -18,13 +18,11 @@
     <sheet name="HeroAcitveSkill" sheetId="16" r:id="rId3"/>
     <sheet name="HeroPassiveSkill" sheetId="17" r:id="rId4"/>
     <sheet name="HeroTranscendSkill" sheetId="9" r:id="rId5"/>
-    <sheet name="NomalEnemy" sheetId="3" r:id="rId6"/>
-    <sheet name="EliteEnemy" sheetId="13" r:id="rId7"/>
-    <sheet name="BossEnemy" sheetId="14" r:id="rId8"/>
-    <sheet name="DropItem" sheetId="4" r:id="rId9"/>
-    <sheet name="Equipment" sheetId="5" r:id="rId10"/>
-    <sheet name="Stage" sheetId="12" r:id="rId11"/>
-    <sheet name="Wave" sheetId="15" r:id="rId12"/>
+    <sheet name="Enemy" sheetId="3" r:id="rId6"/>
+    <sheet name="DropItem" sheetId="4" r:id="rId7"/>
+    <sheet name="Equipment" sheetId="5" r:id="rId8"/>
+    <sheet name="Stage" sheetId="12" r:id="rId9"/>
+    <sheet name="Wave" sheetId="15" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="249">
   <si>
     <t>Index</t>
   </si>
@@ -254,52 +252,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>일반</t>
-  </si>
-  <si>
-    <t>정예</t>
-  </si>
-  <si>
-    <t>닭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>쥐</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>곰</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑우</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>다크바니</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_chicken</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_mouse</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_bear</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_blackCow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_darkBunny</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>죽음의 연꽃</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -334,18 +286,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>_enemy_chickenKing</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>꼬꼬킹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ground</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Wind</t>
   </si>
   <si>
@@ -353,26 +293,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Dark</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Type</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>일반</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보스</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>정예</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>기본체력</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -403,57 +327,6 @@
   <si>
     <t>Boss Enemy</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>_enemy_snake</t>
-  </si>
-  <si>
-    <t>뱀</t>
-  </si>
-  <si>
-    <t>Earth</t>
-  </si>
-  <si>
-    <t>_enemy_crow</t>
-  </si>
-  <si>
-    <t>까마귀</t>
-  </si>
-  <si>
-    <t>_enemy_boar</t>
-  </si>
-  <si>
-    <t>멧돼지</t>
-  </si>
-  <si>
-    <t>_enemy_frog</t>
-  </si>
-  <si>
-    <t>개구리</t>
-  </si>
-  <si>
-    <t>_enemy_scorpion</t>
-  </si>
-  <si>
-    <t>전갈</t>
-  </si>
-  <si>
-    <t>_enemy_wolf</t>
-  </si>
-  <si>
-    <t>늑대</t>
-  </si>
-  <si>
-    <t>_enemy_crocodile</t>
-  </si>
-  <si>
-    <t>악어</t>
-  </si>
-  <si>
-    <t>_enemy_golem</t>
-  </si>
-  <si>
-    <t>골렘</t>
   </si>
   <si>
     <t>골드</t>
@@ -874,6 +747,162 @@
 정예 적 처치시, 반드시 3개를 드롭
 보스 처치시, 반드시 5개를 드롭</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Normal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_normal</t>
+  </si>
+  <si>
+    <t>_enemy_normal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_normalBow</t>
+  </si>
+  <si>
+    <t>_enemy_normalBow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_normal1</t>
+  </si>
+  <si>
+    <t>_enemy_normal1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_normalRush</t>
+  </si>
+  <si>
+    <t>_enemy_normalRush</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_elite</t>
+  </si>
+  <si>
+    <t>_enemy_elite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_elite1</t>
+  </si>
+  <si>
+    <t>_enemy_elite1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_eliteBow</t>
+  </si>
+  <si>
+    <t>_enemy_eliteBow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_eliteRush</t>
+  </si>
+  <si>
+    <t>_enemy_eliteRush</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_boss</t>
+  </si>
+  <si>
+    <t>_enemy_boss</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_bossRush</t>
+  </si>
+  <si>
+    <t>_enemy_bossRush</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_bossStop</t>
+  </si>
+  <si>
+    <t>_enemy_bossStop</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>_enemy_bossBow</t>
+  </si>
+  <si>
+    <t>_enemy_bossBow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>돌진예열시간</t>
+  </si>
+  <si>
+    <t>돌진예열시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>돌진시간</t>
+  </si>
+  <si>
+    <t>돌진시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅감지거리</t>
+  </si>
+  <si>
+    <t>영웅감지거리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스킬쿨타임</t>
+  </si>
+  <si>
+    <t>스킬쿨타임</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스킬시전시간</t>
+  </si>
+  <si>
+    <t>스킬시전시간</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>로컬라이징용 키값</t>
+  </si>
+  <si>
+    <t>이름</t>
+  </si>
+  <si>
+    <t>속성</t>
+  </si>
+  <si>
+    <t>타입</t>
+  </si>
+  <si>
+    <t>기본체력</t>
+  </si>
+  <si>
+    <t>기본공격력</t>
+  </si>
+  <si>
+    <t>이동속도</t>
+  </si>
+  <si>
+    <t>(빈칸)</t>
+  </si>
+  <si>
+    <t>Elite</t>
+  </si>
+  <si>
+    <t>Boss</t>
   </si>
 </sst>
 </file>
@@ -1297,269 +1326,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC93D29-8092-4F32-B3C5-0324AF618AAF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A800D66D-8D9E-44A6-95C2-7A226360B740}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.75" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H1" t="s">
-        <v>139</v>
-      </c>
-      <c r="I1" t="s">
-        <v>147</v>
-      </c>
-      <c r="J1" t="s">
-        <v>149</v>
-      </c>
-      <c r="K1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G2" t="s">
-        <v>95</v>
-      </c>
-      <c r="H2" t="s">
-        <v>140</v>
-      </c>
-      <c r="I2" t="s">
-        <v>148</v>
-      </c>
-      <c r="J2" t="s">
-        <v>150</v>
-      </c>
-      <c r="K2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>480</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" t="s">
-        <v>133</v>
-      </c>
-      <c r="F5" t="s">
-        <v>138</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>480</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" t="s">
-        <v>131</v>
-      </c>
-      <c r="E6" t="s">
-        <v>129</v>
-      </c>
-      <c r="F6" t="s">
-        <v>138</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>480</v>
-      </c>
-      <c r="I6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" t="s">
-        <v>145</v>
-      </c>
-      <c r="D7" t="s">
-        <v>146</v>
-      </c>
-      <c r="E7" t="s">
-        <v>129</v>
-      </c>
-      <c r="F7" t="s">
-        <v>138</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
-        <v>152</v>
-      </c>
-      <c r="K7">
-        <v>600</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2904E33-FA20-49EB-A37A-8A59B5E55789}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1580,49 +1346,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="B1" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="C1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E1" t="s">
+        <v>165</v>
+      </c>
+      <c r="F1" t="s">
+        <v>166</v>
+      </c>
+      <c r="G1" t="s">
+        <v>167</v>
+      </c>
+      <c r="H1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I1" t="s">
+        <v>169</v>
+      </c>
+      <c r="J1" t="s">
+        <v>170</v>
+      </c>
+      <c r="K1" t="s">
+        <v>171</v>
+      </c>
+      <c r="L1" t="s">
+        <v>172</v>
+      </c>
+      <c r="M1" t="s">
+        <v>173</v>
+      </c>
+      <c r="N1" t="s">
         <v>174</v>
       </c>
-      <c r="D1" t="s">
-        <v>200</v>
-      </c>
-      <c r="E1" t="s">
-        <v>201</v>
-      </c>
-      <c r="F1" t="s">
-        <v>202</v>
-      </c>
-      <c r="G1" t="s">
-        <v>203</v>
-      </c>
-      <c r="H1" t="s">
-        <v>204</v>
-      </c>
-      <c r="I1" t="s">
-        <v>205</v>
-      </c>
-      <c r="J1" t="s">
-        <v>206</v>
-      </c>
-      <c r="K1" t="s">
-        <v>207</v>
-      </c>
-      <c r="L1" t="s">
-        <v>208</v>
-      </c>
-      <c r="M1" t="s">
-        <v>209</v>
-      </c>
-      <c r="N1" t="s">
-        <v>210</v>
-      </c>
       <c r="O1" t="s">
-        <v>211</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -1630,10 +1396,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>212</v>
+        <v>176</v>
       </c>
       <c r="C2" t="s">
-        <v>213</v>
+        <v>177</v>
       </c>
       <c r="D2">
         <v>200</v>
@@ -1677,10 +1443,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>178</v>
       </c>
       <c r="C3" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="D3">
         <v>200</v>
@@ -1732,10 +1498,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="B1" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
@@ -1747,34 +1513,34 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
-        <v>165</v>
+        <v>129</v>
       </c>
       <c r="G1" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
       <c r="H1" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="I1" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="J1" t="s">
-        <v>157</v>
+        <v>121</v>
       </c>
       <c r="K1" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="L1" t="s">
-        <v>170</v>
+        <v>134</v>
       </c>
       <c r="M1" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="N1" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="O1" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="P1" t="s">
         <v>15</v>
@@ -1791,7 +1557,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -1839,7 +1605,7 @@
         <v>23</v>
       </c>
       <c r="R2" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -1847,7 +1613,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -1895,7 +1661,7 @@
         <v>23</v>
       </c>
       <c r="R3" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -1903,7 +1669,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -1951,7 +1717,7 @@
         <v>23</v>
       </c>
       <c r="R4" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -1959,7 +1725,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -2007,7 +1773,7 @@
         <v>23</v>
       </c>
       <c r="R5" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
@@ -2015,7 +1781,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -2063,7 +1829,7 @@
         <v>23</v>
       </c>
       <c r="R6" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
@@ -2119,7 +1885,7 @@
         <v>23</v>
       </c>
       <c r="R7" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -2175,7 +1941,7 @@
         <v>23</v>
       </c>
       <c r="R8" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
@@ -2231,7 +1997,7 @@
         <v>23</v>
       </c>
       <c r="R9" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
@@ -2287,7 +2053,7 @@
         <v>23</v>
       </c>
       <c r="R10" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -2343,7 +2109,7 @@
         <v>23</v>
       </c>
       <c r="R11" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
@@ -2399,7 +2165,7 @@
         <v>23</v>
       </c>
       <c r="R12" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -2455,7 +2221,7 @@
         <v>23</v>
       </c>
       <c r="R13" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
@@ -2511,7 +2277,7 @@
         <v>23</v>
       </c>
       <c r="R14" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
@@ -2567,7 +2333,7 @@
         <v>23</v>
       </c>
       <c r="R15" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
@@ -2623,7 +2389,7 @@
         <v>23</v>
       </c>
       <c r="R16" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -2634,7 +2400,7 @@
         <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2679,7 +2445,7 @@
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -2690,7 +2456,7 @@
         <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2735,7 +2501,7 @@
         <v>23</v>
       </c>
       <c r="R18" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -2746,7 +2512,7 @@
         <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -2791,7 +2557,7 @@
         <v>23</v>
       </c>
       <c r="R19" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
@@ -2802,7 +2568,7 @@
         <v>47</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="D20">
         <v>4</v>
@@ -2847,7 +2613,7 @@
         <v>23</v>
       </c>
       <c r="R20" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
@@ -2858,7 +2624,7 @@
         <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="D21">
         <v>5</v>
@@ -2903,7 +2669,7 @@
         <v>23</v>
       </c>
       <c r="R21" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
@@ -2911,10 +2677,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C22" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2959,7 +2725,7 @@
         <v>23</v>
       </c>
       <c r="R22" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
@@ -2967,10 +2733,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C23" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="D23">
         <v>2</v>
@@ -3015,7 +2781,7 @@
         <v>23</v>
       </c>
       <c r="R23" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
@@ -3023,10 +2789,10 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C24" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -3071,7 +2837,7 @@
         <v>23</v>
       </c>
       <c r="R24" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
@@ -3079,10 +2845,10 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C25" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -3127,7 +2893,7 @@
         <v>23</v>
       </c>
       <c r="R25" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
@@ -3135,10 +2901,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C26" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -3183,7 +2949,7 @@
         <v>23</v>
       </c>
       <c r="R26" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -3208,10 +2974,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>5</v>
@@ -3220,10 +2986,10 @@
         <v>4</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>220</v>
+        <v>184</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>14</v>
@@ -3234,22 +3000,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="D2" s="7">
         <v>1</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="F2" s="7">
         <v>0.2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -3257,22 +3023,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="D3" s="7">
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="F3" s="7">
         <v>0.4</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3280,22 +3046,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="D4" s="7">
         <v>3</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="F4" s="7">
         <v>0.6</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3303,22 +3069,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="D5" s="7">
         <v>4</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="F5" s="7">
         <v>0.8</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3326,22 +3092,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="D6" s="7">
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3349,22 +3115,22 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="D7" s="7">
         <v>1</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="F7" s="7">
         <v>0.2</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3372,22 +3138,22 @@
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="D8" s="7">
         <v>2</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="F8" s="7">
         <v>0.4</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3395,22 +3161,22 @@
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="D9" s="7">
         <v>3</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="F9" s="7">
         <v>0.6</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3418,22 +3184,22 @@
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="D10" s="7">
         <v>4</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="F10" s="7">
         <v>0.8</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3441,22 +3207,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="D11" s="7">
         <v>5</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="F11" s="7">
         <v>1</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3464,22 +3230,22 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D12" s="7">
         <v>1</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F12" s="7">
         <v>0.2</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -3487,22 +3253,22 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D13" s="7">
         <v>2</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F13" s="7">
         <v>0.4</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -3510,22 +3276,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D14" s="7">
         <v>3</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F14" s="7">
         <v>0.6</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -3533,22 +3299,22 @@
         <v>3</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D15" s="7">
         <v>4</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F15" s="7">
         <v>0.8</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -3556,22 +3322,22 @@
         <v>3</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D16" s="7">
         <v>5</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="F16" s="7">
         <v>1</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -3579,10 +3345,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="D17" s="7">
         <v>1</v>
@@ -3594,7 +3360,7 @@
         <v>0.2</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -3602,10 +3368,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="D18" s="7">
         <v>2</v>
@@ -3617,7 +3383,7 @@
         <v>0.4</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -3625,10 +3391,10 @@
         <v>4</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="D19" s="7">
         <v>3</v>
@@ -3640,7 +3406,7 @@
         <v>0.6</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -3648,10 +3414,10 @@
         <v>4</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="D20" s="7">
         <v>4</v>
@@ -3663,7 +3429,7 @@
         <v>0.8</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -3671,10 +3437,10 @@
         <v>4</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="D21" s="7">
         <v>5</v>
@@ -3686,7 +3452,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -3941,7 +3707,7 @@
         <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -3980,7 +3746,7 @@
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -4012,7 +3778,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E98403FE-290B-485A-ADFB-39718B202EA0}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
@@ -4024,7 +3790,7 @@
     <col min="8" max="8" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -4035,22 +3801,37 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" t="s">
         <v>71</v>
-      </c>
-      <c r="F1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G1" t="s">
-        <v>90</v>
       </c>
       <c r="H1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" t="s">
+        <v>230</v>
+      </c>
+      <c r="J1" t="s">
+        <v>232</v>
+      </c>
+      <c r="K1" t="s">
+        <v>234</v>
+      </c>
+      <c r="L1" t="s">
+        <v>236</v>
+      </c>
+      <c r="M1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -4061,22 +3842,22 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="F2" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -4102,389 +3883,806 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
+        <v>206</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F4">
+        <v>204</v>
+      </c>
+      <c r="F4" s="1">
         <v>50</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>10</v>
       </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H4" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>210</v>
+      </c>
+      <c r="D5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E5" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5">
-        <v>30</v>
-      </c>
-      <c r="G5">
+      <c r="F5" s="1">
+        <v>55</v>
+      </c>
+      <c r="G5" s="1">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1">
+        <v>8</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
         <v>10</v>
       </c>
-      <c r="H5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" s="1">
-        <v>45</v>
-      </c>
-      <c r="G6" s="1">
-        <v>12</v>
-      </c>
-      <c r="H6" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>57</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
       <c r="F7" s="1">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G7" s="1">
         <v>15</v>
       </c>
       <c r="H7" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>85</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
       <c r="F8" s="1">
-        <v>60</v>
+        <v>1000</v>
       </c>
       <c r="G8" s="1">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="H8" s="1">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>85</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
       <c r="F9" s="1">
-        <v>40</v>
+        <v>1200</v>
       </c>
       <c r="G9" s="1">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="H9" s="1">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>85</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
       <c r="F10" s="1">
+        <v>900</v>
+      </c>
+      <c r="G10" s="1">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="J10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>220</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1100</v>
+      </c>
+      <c r="G11" s="1">
+        <v>38</v>
+      </c>
+      <c r="H11" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G12" s="1">
+        <v>100</v>
+      </c>
+      <c r="H12" s="1">
+        <v>5</v>
+      </c>
+      <c r="L12">
+        <v>10</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>3</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G13" s="1">
+        <v>150</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>4</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1">
+        <v>15500</v>
+      </c>
+      <c r="G14" s="1">
+        <v>120</v>
+      </c>
+      <c r="H14" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>228</v>
+      </c>
+      <c r="F15" s="1">
+        <v>14000</v>
+      </c>
+      <c r="G15" s="1">
+        <v>90</v>
+      </c>
+      <c r="H15" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="K15">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>1</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F18" s="1">
+        <v>50</v>
+      </c>
+      <c r="G18" s="1">
+        <v>10</v>
+      </c>
+      <c r="H18" s="1">
+        <v>3</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="K18" s="1">
+        <v>5</v>
+      </c>
+      <c r="L18" s="1">
+        <v>8</v>
+      </c>
+      <c r="M18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>2</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F19" s="1">
         <v>55</v>
       </c>
-      <c r="G10" s="1">
-        <v>14</v>
-      </c>
-      <c r="H10" s="1">
+      <c r="G19" s="1">
+        <v>12</v>
+      </c>
+      <c r="H19" s="1">
+        <v>3</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J19" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="K19" s="1">
+        <v>5</v>
+      </c>
+      <c r="L19" s="1">
+        <v>8</v>
+      </c>
+      <c r="M19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>3</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F20" s="1">
+        <v>40</v>
+      </c>
+      <c r="G20" s="1">
+        <v>8</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I20" s="1">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1">
+        <v>1</v>
+      </c>
+      <c r="K20" s="1">
+        <v>10</v>
+      </c>
+      <c r="L20" s="1">
+        <v>6</v>
+      </c>
+      <c r="M20" s="1">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>4</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F21" s="1">
+        <v>60</v>
+      </c>
+      <c r="G21" s="1">
+        <v>15</v>
+      </c>
+      <c r="H21" s="1">
         <v>3.5</v>
       </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75EDD00F-7CC0-430A-8135-8AD1CC82CF89}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I21" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="K21" s="1">
+        <v>6</v>
+      </c>
+      <c r="L21" s="1">
+        <v>10</v>
+      </c>
+      <c r="M21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>5</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1000</v>
+      </c>
+      <c r="G22" s="1">
+        <v>30</v>
+      </c>
+      <c r="H22" s="1">
+        <v>4</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="K22" s="1">
+        <v>8</v>
+      </c>
+      <c r="L22" s="1">
+        <v>12</v>
+      </c>
+      <c r="M22" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>6</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1200</v>
+      </c>
+      <c r="G23" s="1">
+        <v>35</v>
+      </c>
+      <c r="H23" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="I23" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="J23" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="K23" s="1">
+        <v>8</v>
+      </c>
+      <c r="L23" s="1">
+        <v>12</v>
+      </c>
+      <c r="M23" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>7</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F24" s="1">
+        <v>900</v>
+      </c>
+      <c r="G24" s="1">
+        <v>28</v>
+      </c>
+      <c r="H24" s="1">
+        <v>1</v>
+      </c>
+      <c r="I24" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J24" s="1">
+        <v>1</v>
+      </c>
+      <c r="K24" s="1">
+        <v>12</v>
+      </c>
+      <c r="L24" s="1">
+        <v>10</v>
+      </c>
+      <c r="M24" s="1">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>8</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F25" s="1">
+        <v>1100</v>
+      </c>
+      <c r="G25" s="1">
+        <v>38</v>
+      </c>
+      <c r="H25" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="I25" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="J25" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="K25" s="1">
+        <v>7</v>
+      </c>
+      <c r="L25" s="1">
+        <v>10</v>
+      </c>
+      <c r="M25" s="1">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>9</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F26" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G26" s="1">
+        <v>100</v>
+      </c>
+      <c r="H26" s="1">
+        <v>5</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1</v>
+      </c>
+      <c r="J26" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="K26" s="1">
+        <v>15</v>
+      </c>
+      <c r="L26" s="1">
+        <v>10</v>
+      </c>
+      <c r="M26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>10</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F27" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27" s="1">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1">
+        <v>0</v>
+      </c>
+      <c r="M27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>11</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F28" s="1">
+        <v>15500</v>
+      </c>
+      <c r="G28" s="1">
+        <v>120</v>
+      </c>
+      <c r="H28" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="I28" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J28" s="1">
+        <v>2</v>
+      </c>
+      <c r="K28" s="1">
+        <v>15</v>
+      </c>
+      <c r="L28" s="1">
+        <v>8</v>
+      </c>
+      <c r="M28" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>12</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F29" s="1">
+        <v>14000</v>
+      </c>
+      <c r="G29" s="1">
         <v>90</v>
       </c>
-      <c r="H1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="H29" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="I29" s="1">
+        <v>1</v>
+      </c>
+      <c r="J29" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="K29" s="1">
+        <v>20</v>
+      </c>
+      <c r="L29" s="1">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4">
-        <v>200</v>
-      </c>
-      <c r="G4">
-        <v>20</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="1">
-        <v>180</v>
-      </c>
-      <c r="G5" s="1">
-        <v>22</v>
-      </c>
-      <c r="H5" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="1">
-        <v>220</v>
-      </c>
-      <c r="G6" s="1">
-        <v>24</v>
-      </c>
-      <c r="H6" s="1">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" s="1">
-        <v>300</v>
-      </c>
-      <c r="G7" s="1">
-        <v>30</v>
-      </c>
-      <c r="H7" s="1">
-        <v>2.5</v>
+      <c r="M29" s="1">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -4494,184 +4692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D449D71E-9D1D-4FE4-BD05-A6B5ADA27DE6}">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4">
-        <v>1000</v>
-      </c>
-      <c r="G4">
-        <v>50</v>
-      </c>
-      <c r="H4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" t="s">
-        <v>86</v>
-      </c>
-      <c r="F5">
-        <v>3000</v>
-      </c>
-      <c r="G5">
-        <v>80</v>
-      </c>
-      <c r="H5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6">
-        <v>5000</v>
-      </c>
-      <c r="G6">
-        <v>100</v>
-      </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90154975-8943-4FC8-832E-3EF623D7F44A}">
   <dimension ref="A1:M20"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -4692,40 +4713,40 @@
   <sheetData>
     <row r="1" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>192</v>
-      </c>
       <c r="E1" s="5" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>196</v>
+        <v>160</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>197</v>
+        <v>161</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>198</v>
+        <v>162</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>199</v>
+        <v>163</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>14</v>
@@ -4736,10 +4757,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="D2" s="1">
         <v>5</v>
@@ -4751,13 +4772,13 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1" t="s">
-        <v>238</v>
+        <v>202</v>
       </c>
       <c r="L2" s="1">
         <v>100</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4765,10 +4786,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1">
@@ -4780,11 +4801,11 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1" t="s">
-        <v>237</v>
+        <v>201</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -4792,10 +4813,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -4807,13 +4828,13 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="L4" s="1">
         <v>100</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>185</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -4821,10 +4842,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>123</v>
+        <v>87</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4833,16 +4854,16 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="L5" s="1">
         <v>1</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -4850,10 +4871,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -4867,13 +4888,13 @@
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="L6" s="1">
         <v>1</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4881,10 +4902,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -4896,13 +4917,13 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>236</v>
+        <v>200</v>
       </c>
       <c r="L7" s="1">
         <v>1</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>188</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -4910,10 +4931,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -4922,16 +4943,16 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="L8" s="1">
         <v>1</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
@@ -4939,10 +4960,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>178</v>
+        <v>142</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -4951,14 +4972,14 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>179</v>
+        <v>143</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>191</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -5084,4 +5105,267 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC93D29-8092-4F32-B3C5-0324AF618AAF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A800D66D-8D9E-44A6-95C2-7A226360B740}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>480</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>480</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>480</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K7">
+        <v>600</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add intro and play scenes, refactor enemy and bullet logic
Introduced new scenes (00_Intro, 02_Play), updated main scene UI, and reorganized shop scene. Added ranged attack enemy logic, new bullet handling (including EnemyArrow and HeroBullet), and refactored bullet code into a generic location. Updated prefabs and data assets to support new enemy and skill types, and made related changes to scripts and managers for improved modularity and maintainability.
</commit_message>
<xml_diff>
--- a/Assets/DataTable.xlsx
+++ b/Assets/DataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\KSSStudy\Projects\TangTang\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8090F2B2-A653-4229-ABEA-647A02425854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A06C6B-70EB-4126-BF50-1566E932EAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="709" activeTab="5" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
+    <workbookView xWindow="4455" yWindow="4185" windowWidth="21600" windowHeight="11295" tabRatio="709" firstSheet="3" activeTab="7" xr2:uid="{760CB9A7-C303-4CC0-8C81-37FBE4BECC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Player" sheetId="6" r:id="rId1"/>
@@ -19,10 +19,13 @@
     <sheet name="HeroPassiveSkill" sheetId="17" r:id="rId4"/>
     <sheet name="HeroTranscendSkill" sheetId="9" r:id="rId5"/>
     <sheet name="Enemy" sheetId="3" r:id="rId6"/>
-    <sheet name="DropItem" sheetId="4" r:id="rId7"/>
-    <sheet name="Equipment" sheetId="5" r:id="rId8"/>
-    <sheet name="Stage" sheetId="12" r:id="rId9"/>
-    <sheet name="Wave" sheetId="15" r:id="rId10"/>
+    <sheet name="RushEnemy" sheetId="18" r:id="rId7"/>
+    <sheet name="RangedAttackEnemy" sheetId="19" r:id="rId8"/>
+    <sheet name="SkillEnemy" sheetId="20" r:id="rId9"/>
+    <sheet name="DropItem" sheetId="4" r:id="rId10"/>
+    <sheet name="Equipment" sheetId="5" r:id="rId11"/>
+    <sheet name="Stage" sheetId="12" r:id="rId12"/>
+    <sheet name="Wave" sheetId="15" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="229">
   <si>
     <t>Index</t>
   </si>
@@ -203,10 +206,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>이동속도</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>_heroActiveSkill_dragonBall</t>
   </si>
   <si>
@@ -260,36 +259,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>타입</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>속성</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Element</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Fire</t>
-  </si>
-  <si>
-    <t>Fire</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Water</t>
-  </si>
-  <si>
-    <t>Water</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Wind</t>
-  </si>
-  <si>
-    <t>Wind</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -297,15 +279,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>기본체력</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>BaseMaxHp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>기본공격력</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -750,170 +724,138 @@
   </si>
   <si>
     <t>Normal</t>
-  </si>
-  <si>
-    <t>Normal</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_normal</t>
-  </si>
-  <si>
-    <t>_enemy_normal</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_normalBow</t>
-  </si>
-  <si>
-    <t>_enemy_normalBow</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_normal1</t>
-  </si>
-  <si>
-    <t>_enemy_normal1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_normalRush</t>
-  </si>
-  <si>
-    <t>_enemy_normalRush</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_elite</t>
-  </si>
-  <si>
-    <t>_enemy_elite</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_elite1</t>
-  </si>
-  <si>
-    <t>_enemy_elite1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_eliteBow</t>
-  </si>
-  <si>
-    <t>_enemy_eliteBow</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_eliteRush</t>
-  </si>
-  <si>
-    <t>_enemy_eliteRush</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_boss</t>
-  </si>
-  <si>
-    <t>_enemy_boss</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_bossRush</t>
-  </si>
-  <si>
-    <t>_enemy_bossRush</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_bossStop</t>
-  </si>
-  <si>
-    <t>_enemy_bossStop</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>_enemy_bossBow</t>
-  </si>
-  <si>
-    <t>_enemy_bossBow</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌진예열시간</t>
-  </si>
-  <si>
-    <t>돌진예열시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌진시간</t>
-  </si>
-  <si>
-    <t>돌진시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>영웅감지거리</t>
-  </si>
-  <si>
-    <t>영웅감지거리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스킬쿨타임</t>
-  </si>
-  <si>
-    <t>스킬쿨타임</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>스킬시전시간</t>
-  </si>
-  <si>
-    <t>스킬시전시간</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>로컬라이징용 키값</t>
-  </si>
-  <si>
-    <t>이름</t>
-  </si>
-  <si>
-    <t>속성</t>
-  </si>
-  <si>
-    <t>타입</t>
-  </si>
-  <si>
-    <t>기본체력</t>
-  </si>
-  <si>
-    <t>기본공격력</t>
-  </si>
-  <si>
-    <t>이동속도</t>
-  </si>
-  <si>
-    <t>(빈칸)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RushCoolTime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ReadyDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RushDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RushSpeed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SkillCoolTime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SkillReadyDuration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반원거리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일반돌진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엘리트</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엘리트1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엘리트원거리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엘리트돌진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스돌진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스고정</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>보스원거리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Elite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Boss</t>
-  </si>
-  <si>
-    <t>돌진속도</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌진쿨타임</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>원거리공격쿨타임</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AttackSpan</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1338,6 +1280,684 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90154975-8943-4FC8-832E-3EF623D7F44A}">
+  <dimension ref="A1:M20"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="18.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="56.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="1">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="L2" s="1">
+        <v>100</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1">
+        <v>5</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L4" s="1">
+        <v>100</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>10</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC93D29-8092-4F32-B3C5-0324AF618AAF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A800D66D-8D9E-44A6-95C2-7A226360B740}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J1" t="s">
+        <v>105</v>
+      </c>
+      <c r="K1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I2" t="s">
+        <v>104</v>
+      </c>
+      <c r="J2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>480</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>480</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>480</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F7" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>108</v>
+      </c>
+      <c r="K7">
+        <v>600</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2904E33-FA20-49EB-A37A-8A59B5E55789}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1358,49 +1978,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H1" t="s">
+        <v>160</v>
+      </c>
+      <c r="I1" t="s">
+        <v>161</v>
+      </c>
+      <c r="J1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L1" t="s">
         <v>164</v>
       </c>
-      <c r="E1" t="s">
+      <c r="M1" t="s">
         <v>165</v>
       </c>
-      <c r="F1" t="s">
+      <c r="N1" t="s">
         <v>166</v>
       </c>
-      <c r="G1" t="s">
+      <c r="O1" t="s">
         <v>167</v>
-      </c>
-      <c r="H1" t="s">
-        <v>168</v>
-      </c>
-      <c r="I1" t="s">
-        <v>169</v>
-      </c>
-      <c r="J1" t="s">
-        <v>170</v>
-      </c>
-      <c r="K1" t="s">
-        <v>171</v>
-      </c>
-      <c r="L1" t="s">
-        <v>172</v>
-      </c>
-      <c r="M1" t="s">
-        <v>173</v>
-      </c>
-      <c r="N1" t="s">
-        <v>174</v>
-      </c>
-      <c r="O1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -1408,10 +2028,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="D2">
         <v>200</v>
@@ -1455,10 +2075,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D3">
         <v>200</v>
@@ -1510,10 +2130,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
@@ -1525,34 +2145,34 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>125</v>
+      </c>
+      <c r="L1" t="s">
+        <v>126</v>
+      </c>
+      <c r="M1" t="s">
+        <v>127</v>
+      </c>
+      <c r="N1" t="s">
+        <v>128</v>
+      </c>
+      <c r="O1" t="s">
         <v>129</v>
-      </c>
-      <c r="G1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" t="s">
-        <v>131</v>
-      </c>
-      <c r="I1" t="s">
-        <v>132</v>
-      </c>
-      <c r="J1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K1" t="s">
-        <v>133</v>
-      </c>
-      <c r="L1" t="s">
-        <v>134</v>
-      </c>
-      <c r="M1" t="s">
-        <v>135</v>
-      </c>
-      <c r="N1" t="s">
-        <v>136</v>
-      </c>
-      <c r="O1" t="s">
-        <v>137</v>
       </c>
       <c r="P1" t="s">
         <v>15</v>
@@ -1569,7 +2189,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -1617,7 +2237,7 @@
         <v>23</v>
       </c>
       <c r="R2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -1625,7 +2245,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -1673,7 +2293,7 @@
         <v>23</v>
       </c>
       <c r="R3" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -1681,7 +2301,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -1729,7 +2349,7 @@
         <v>23</v>
       </c>
       <c r="R4" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -1737,7 +2357,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
@@ -1785,7 +2405,7 @@
         <v>23</v>
       </c>
       <c r="R5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
@@ -1793,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -1841,7 +2461,7 @@
         <v>23</v>
       </c>
       <c r="R6" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
@@ -1849,7 +2469,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>
@@ -1897,7 +2517,7 @@
         <v>23</v>
       </c>
       <c r="R7" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -1905,7 +2525,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -1953,7 +2573,7 @@
         <v>23</v>
       </c>
       <c r="R8" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
@@ -1961,7 +2581,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -2009,7 +2629,7 @@
         <v>23</v>
       </c>
       <c r="R9" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
@@ -2017,7 +2637,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>24</v>
@@ -2065,7 +2685,7 @@
         <v>23</v>
       </c>
       <c r="R10" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -2073,7 +2693,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
@@ -2121,7 +2741,7 @@
         <v>23</v>
       </c>
       <c r="R11" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
@@ -2129,7 +2749,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>25</v>
@@ -2177,7 +2797,7 @@
         <v>23</v>
       </c>
       <c r="R12" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -2185,7 +2805,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
         <v>25</v>
@@ -2233,7 +2853,7 @@
         <v>23</v>
       </c>
       <c r="R13" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
@@ -2241,7 +2861,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
         <v>25</v>
@@ -2289,7 +2909,7 @@
         <v>23</v>
       </c>
       <c r="R14" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
@@ -2297,7 +2917,7 @@
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
         <v>25</v>
@@ -2345,7 +2965,7 @@
         <v>23</v>
       </c>
       <c r="R15" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
@@ -2353,7 +2973,7 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
         <v>25</v>
@@ -2401,7 +3021,7 @@
         <v>23</v>
       </c>
       <c r="R16" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -2409,10 +3029,10 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2457,7 +3077,7 @@
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -2465,10 +3085,10 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2513,7 +3133,7 @@
         <v>23</v>
       </c>
       <c r="R18" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -2521,10 +3141,10 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -2569,7 +3189,7 @@
         <v>23</v>
       </c>
       <c r="R19" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
@@ -2577,10 +3197,10 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D20">
         <v>4</v>
@@ -2625,7 +3245,7 @@
         <v>23</v>
       </c>
       <c r="R20" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
@@ -2633,10 +3253,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D21">
         <v>5</v>
@@ -2681,7 +3301,7 @@
         <v>23</v>
       </c>
       <c r="R21" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
@@ -2689,10 +3309,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C22" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2737,7 +3357,7 @@
         <v>23</v>
       </c>
       <c r="R22" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
@@ -2745,10 +3365,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C23" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D23">
         <v>2</v>
@@ -2793,7 +3413,7 @@
         <v>23</v>
       </c>
       <c r="R23" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
@@ -2801,10 +3421,10 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C24" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -2849,7 +3469,7 @@
         <v>23</v>
       </c>
       <c r="R24" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
@@ -2857,10 +3477,10 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C25" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -2905,7 +3525,7 @@
         <v>23</v>
       </c>
       <c r="R25" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
@@ -2913,10 +3533,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -2961,7 +3581,7 @@
         <v>23</v>
       </c>
       <c r="R26" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2986,10 +3606,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>5</v>
@@ -2998,10 +3618,10 @@
         <v>4</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>14</v>
@@ -3012,22 +3632,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D2" s="7">
         <v>1</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F2" s="7">
         <v>0.2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -3035,22 +3655,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D3" s="7">
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F3" s="7">
         <v>0.4</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -3058,22 +3678,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D4" s="7">
         <v>3</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F4" s="7">
         <v>0.6</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -3081,22 +3701,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D5" s="7">
         <v>4</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F5" s="7">
         <v>0.8</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3104,22 +3724,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D6" s="7">
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -3127,22 +3747,22 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D7" s="7">
         <v>1</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F7" s="7">
         <v>0.2</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -3150,22 +3770,22 @@
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D8" s="7">
         <v>2</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F8" s="7">
         <v>0.4</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -3173,22 +3793,22 @@
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D9" s="7">
         <v>3</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F9" s="7">
         <v>0.6</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -3196,22 +3816,22 @@
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D10" s="7">
         <v>4</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F10" s="7">
         <v>0.8</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -3219,22 +3839,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D11" s="7">
         <v>5</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F11" s="7">
         <v>1</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -3242,22 +3862,22 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D12" s="7">
         <v>1</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F12" s="7">
         <v>0.2</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -3265,22 +3885,22 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D13" s="7">
         <v>2</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F13" s="7">
         <v>0.4</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -3288,22 +3908,22 @@
         <v>3</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D14" s="7">
         <v>3</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F14" s="7">
         <v>0.6</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -3311,22 +3931,22 @@
         <v>3</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D15" s="7">
         <v>4</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F15" s="7">
         <v>0.8</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -3334,22 +3954,22 @@
         <v>3</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D16" s="7">
         <v>5</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F16" s="7">
         <v>1</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -3357,10 +3977,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D17" s="7">
         <v>1</v>
@@ -3372,7 +3992,7 @@
         <v>0.2</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -3380,10 +4000,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D18" s="7">
         <v>2</v>
@@ -3395,7 +4015,7 @@
         <v>0.4</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -3403,10 +4023,10 @@
         <v>4</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D19" s="7">
         <v>3</v>
@@ -3418,7 +4038,7 @@
         <v>0.6</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -3426,10 +4046,10 @@
         <v>4</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D20" s="7">
         <v>4</v>
@@ -3441,7 +4061,7 @@
         <v>0.8</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -3449,10 +4069,10 @@
         <v>4</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D21" s="7">
         <v>5</v>
@@ -3464,7 +4084,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -3640,10 +4260,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -3669,7 +4289,7 @@
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -3677,10 +4297,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -3708,7 +4328,7 @@
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -3716,10 +4336,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -3747,7 +4367,7 @@
         <v>90</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -3755,10 +4375,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -3790,976 +4410,355 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E98403FE-290B-485A-ADFB-39718B202EA0}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="1">
+        <v>50</v>
+      </c>
+      <c r="G2" s="1">
+        <v>10</v>
+      </c>
+      <c r="H2" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D3" t="s">
         <v>60</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E3" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" s="1">
+        <v>55</v>
+      </c>
+      <c r="G3" s="1">
+        <v>12</v>
+      </c>
+      <c r="H3" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" s="1">
+        <v>40</v>
+      </c>
+      <c r="G4" s="1">
+        <v>8</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D5" t="s">
         <v>59</v>
       </c>
-      <c r="F1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" t="s">
-        <v>250</v>
-      </c>
-      <c r="J1" t="s">
-        <v>230</v>
-      </c>
-      <c r="K1" t="s">
-        <v>232</v>
-      </c>
-      <c r="L1" t="s">
-        <v>249</v>
-      </c>
-      <c r="M1" t="s">
-        <v>251</v>
-      </c>
-      <c r="N1" t="s">
-        <v>234</v>
-      </c>
-      <c r="O1" t="s">
-        <v>236</v>
-      </c>
-      <c r="P1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="E5" t="s">
+        <v>195</v>
+      </c>
+      <c r="F5" s="1">
+        <v>60</v>
+      </c>
+      <c r="G5" s="1">
+        <v>15</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1000</v>
+      </c>
+      <c r="G6" s="1">
+        <v>30</v>
+      </c>
+      <c r="H6" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1200</v>
+      </c>
+      <c r="G7" s="1">
+        <v>35</v>
+      </c>
+      <c r="H7" s="1">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B8" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="1">
+        <v>900</v>
+      </c>
+      <c r="G8" s="1">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1100</v>
+      </c>
+      <c r="G9" s="1">
+        <v>38</v>
+      </c>
+      <c r="H9" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="E10" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="F10" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G10" s="1">
+        <v>100</v>
+      </c>
+      <c r="H10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>3</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="D4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E4" t="s">
-        <v>204</v>
-      </c>
-      <c r="F4" s="1">
-        <v>50</v>
-      </c>
-      <c r="G4" s="1">
-        <v>10</v>
-      </c>
-      <c r="H4" s="1">
-        <v>3</v>
-      </c>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>210</v>
-      </c>
-      <c r="D5" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="1">
-        <v>55</v>
-      </c>
-      <c r="G5" s="1">
-        <v>12</v>
-      </c>
-      <c r="H5" s="1">
-        <v>3</v>
-      </c>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1">
-        <v>40</v>
-      </c>
-      <c r="G6" s="1">
-        <v>8</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="I6" s="1"/>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+      <c r="C11" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="F11" s="1">
+        <v>15000</v>
+      </c>
+      <c r="G11" s="1">
+        <v>150</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
         <v>4</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1">
+      <c r="B12" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D12" t="s">
         <v>60</v>
       </c>
-      <c r="G7" s="1">
-        <v>15</v>
-      </c>
-      <c r="H7" s="1">
-        <v>3.5</v>
-      </c>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="1">
-        <v>30</v>
-      </c>
-      <c r="H8" s="1">
-        <v>4</v>
-      </c>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1">
-        <v>1200</v>
-      </c>
-      <c r="G9" s="1">
-        <v>35</v>
-      </c>
-      <c r="H9" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1">
-        <v>900</v>
-      </c>
-      <c r="G10" s="1">
-        <v>28</v>
-      </c>
-      <c r="H10" s="1">
-        <v>1</v>
-      </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1">
-        <v>0.7</v>
-      </c>
-      <c r="K10" s="1">
-        <v>1</v>
-      </c>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>220</v>
-      </c>
-      <c r="F11" s="1">
-        <v>1100</v>
-      </c>
-      <c r="G11" s="1">
-        <v>38</v>
-      </c>
-      <c r="H11" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>2</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>227</v>
+      </c>
       <c r="F12" s="1">
-        <v>15000</v>
+        <v>15500</v>
       </c>
       <c r="G12" s="1">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="H12" s="1">
-        <v>5</v>
-      </c>
-      <c r="I12" s="1"/>
-      <c r="O12">
-        <v>10</v>
-      </c>
-      <c r="P12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>3</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>227</v>
+      </c>
       <c r="F13" s="1">
-        <v>15000</v>
+        <v>14000</v>
       </c>
       <c r="G13" s="1">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="H13" s="1">
-        <v>0</v>
-      </c>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>4</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1">
-        <v>15500</v>
-      </c>
-      <c r="G14" s="1">
-        <v>120</v>
-      </c>
-      <c r="H14" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1">
-        <v>1</v>
-      </c>
-      <c r="K14" s="1">
-        <v>2</v>
-      </c>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
-        <v>228</v>
-      </c>
-      <c r="F15" s="1">
-        <v>14000</v>
-      </c>
-      <c r="G15" s="1">
-        <v>90</v>
-      </c>
-      <c r="H15" s="1">
         <v>1.5</v>
-      </c>
-      <c r="I15" s="1"/>
-      <c r="N15">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="33" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="P17" s="5" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="33" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
-        <v>1</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F18" s="1">
-        <v>50</v>
-      </c>
-      <c r="G18" s="1">
-        <v>10</v>
-      </c>
-      <c r="H18" s="1">
-        <v>3</v>
-      </c>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="K18" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1">
-        <v>5</v>
-      </c>
-      <c r="O18" s="1">
-        <v>8</v>
-      </c>
-      <c r="P18" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="33" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
-        <v>2</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F19" s="1">
-        <v>55</v>
-      </c>
-      <c r="G19" s="1">
-        <v>12</v>
-      </c>
-      <c r="H19" s="1">
-        <v>3</v>
-      </c>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="K19" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1">
-        <v>5</v>
-      </c>
-      <c r="O19" s="1">
-        <v>8</v>
-      </c>
-      <c r="P19" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="33" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
-        <v>3</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F20" s="1">
-        <v>40</v>
-      </c>
-      <c r="G20" s="1">
-        <v>8</v>
-      </c>
-      <c r="H20" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1">
-        <v>1</v>
-      </c>
-      <c r="K20" s="1">
-        <v>1</v>
-      </c>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1">
-        <v>10</v>
-      </c>
-      <c r="O20" s="1">
-        <v>6</v>
-      </c>
-      <c r="P20" s="1">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="33" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
-        <v>4</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F21" s="1">
-        <v>60</v>
-      </c>
-      <c r="G21" s="1">
-        <v>15</v>
-      </c>
-      <c r="H21" s="1">
-        <v>3.5</v>
-      </c>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="K21" s="1">
-        <v>1.2</v>
-      </c>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1">
-        <v>6</v>
-      </c>
-      <c r="O21" s="1">
-        <v>10</v>
-      </c>
-      <c r="P21" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
-        <v>5</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="F22" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G22" s="1">
-        <v>30</v>
-      </c>
-      <c r="H22" s="1">
-        <v>4</v>
-      </c>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="K22" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1">
-        <v>8</v>
-      </c>
-      <c r="O22" s="1">
-        <v>12</v>
-      </c>
-      <c r="P22" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
-        <v>6</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="F23" s="1">
-        <v>1200</v>
-      </c>
-      <c r="G23" s="1">
-        <v>35</v>
-      </c>
-      <c r="H23" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1">
-        <v>0.6</v>
-      </c>
-      <c r="K23" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1">
-        <v>8</v>
-      </c>
-      <c r="O23" s="1">
-        <v>12</v>
-      </c>
-      <c r="P23" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>7</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="F24" s="1">
-        <v>900</v>
-      </c>
-      <c r="G24" s="1">
-        <v>28</v>
-      </c>
-      <c r="H24" s="1">
-        <v>1</v>
-      </c>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="K24" s="1">
-        <v>1</v>
-      </c>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1">
-        <v>12</v>
-      </c>
-      <c r="O24" s="1">
-        <v>10</v>
-      </c>
-      <c r="P24" s="1">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
-        <v>8</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="F25" s="1">
-        <v>1100</v>
-      </c>
-      <c r="G25" s="1">
-        <v>38</v>
-      </c>
-      <c r="H25" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="K25" s="1">
-        <v>1.4</v>
-      </c>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1">
-        <v>7</v>
-      </c>
-      <c r="O25" s="1">
-        <v>10</v>
-      </c>
-      <c r="P25" s="1">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
-        <v>9</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="F26" s="1">
-        <v>15000</v>
-      </c>
-      <c r="G26" s="1">
-        <v>100</v>
-      </c>
-      <c r="H26" s="1">
-        <v>5</v>
-      </c>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1">
-        <v>1</v>
-      </c>
-      <c r="K26" s="1">
-        <v>2.5</v>
-      </c>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1">
-        <v>15</v>
-      </c>
-      <c r="O26" s="1">
-        <v>10</v>
-      </c>
-      <c r="P26" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A27" s="1">
-        <v>10</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="F27" s="1">
-        <v>15000</v>
-      </c>
-      <c r="G27" s="1">
-        <v>0</v>
-      </c>
-      <c r="H27" s="1">
-        <v>0</v>
-      </c>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1">
-        <v>0</v>
-      </c>
-      <c r="K27" s="1">
-        <v>0</v>
-      </c>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1">
-        <v>0</v>
-      </c>
-      <c r="O27" s="1">
-        <v>0</v>
-      </c>
-      <c r="P27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
-        <v>11</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="F28" s="1">
-        <v>15500</v>
-      </c>
-      <c r="G28" s="1">
-        <v>120</v>
-      </c>
-      <c r="H28" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="K28" s="1">
-        <v>2</v>
-      </c>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1">
-        <v>15</v>
-      </c>
-      <c r="O28" s="1">
-        <v>8</v>
-      </c>
-      <c r="P28" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
-        <v>12</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="F29" s="1">
-        <v>14000</v>
-      </c>
-      <c r="G29" s="1">
-        <v>90</v>
-      </c>
-      <c r="H29" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1">
-        <v>1</v>
-      </c>
-      <c r="K29" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1">
-        <v>20</v>
-      </c>
-      <c r="O29" s="1">
-        <v>12</v>
-      </c>
-      <c r="P29" s="1">
-        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -4770,675 +4769,96 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90154975-8943-4FC8-832E-3EF623D7F44A}">
-  <dimension ref="A1:M20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65607DF9-57A4-47E8-BBE4-C8837F7E8708}">
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="56.75" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" s="1">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L2" s="1">
-        <v>100</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="33" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1">
-        <v>5</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="L4" s="1">
-        <v>100</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="L5" s="1">
-        <v>1</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="I6" s="1">
-        <v>10</v>
-      </c>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="L6" s="1">
-        <v>1</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="33" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="L7" s="1">
-        <v>1</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="L8" s="1">
-        <v>1</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="M11" s="1"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="33" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>205</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC93D29-8092-4F32-B3C5-0324AF618AAF}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E3B05EF-D2FA-4359-BFC8-E88326C444E6}">
+  <dimension ref="C1:K1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A800D66D-8D9E-44A6-95C2-7A226360B740}">
-  <dimension ref="A1:K7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E361376E-45A9-42C9-903C-F3B628704F4A}">
+  <dimension ref="C1:D1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.75" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" t="s">
-        <v>27</v>
-      </c>
+    <row r="1" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C1" t="s">
-        <v>13</v>
+        <v>212</v>
       </c>
       <c r="D1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F1" t="s">
-        <v>100</v>
-      </c>
-      <c r="G1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H1" t="s">
-        <v>103</v>
-      </c>
-      <c r="I1" t="s">
-        <v>111</v>
-      </c>
-      <c r="J1" t="s">
-        <v>113</v>
-      </c>
-      <c r="K1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G2" t="s">
-        <v>76</v>
-      </c>
-      <c r="H2" t="s">
-        <v>104</v>
-      </c>
-      <c r="I2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J2" t="s">
-        <v>114</v>
-      </c>
-      <c r="K2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" t="s">
-        <v>93</v>
-      </c>
-      <c r="E4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>480</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F5" t="s">
-        <v>102</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>480</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" t="s">
-        <v>95</v>
-      </c>
-      <c r="E6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>480</v>
-      </c>
-      <c r="I6" t="b">
-        <v>1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" t="s">
-        <v>93</v>
-      </c>
-      <c r="F7" t="s">
-        <v>102</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
-        <v>116</v>
-      </c>
-      <c r="K7">
-        <v>600</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>